<commit_message>
📊 Consolidated Test Report – Build #2 2a94aded317406ee044c9c2096ff2bca0a2d6297
</commit_message>
<xml_diff>
--- a/backend-reports/functional-test-report.xlsx
+++ b/backend-reports/functional-test-report.xlsx
@@ -83,7 +83,7 @@
     <t>Date &amp; Time</t>
   </si>
   <si>
-    <t>7/19/2026, 5:34:17 PM</t>
+    <t>7/19/2026, 5:56:26 PM</t>
   </si>
   <si>
     <t>Duration</t>
@@ -3373,7 +3373,7 @@
         <v>36</v>
       </c>
       <c r="G2" s="19">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>37</v>
@@ -3399,7 +3399,7 @@
         <v>36</v>
       </c>
       <c r="G3" s="19">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H3" s="17" t="s">
         <v>37</v>
@@ -3425,7 +3425,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="19">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>37</v>
@@ -3451,7 +3451,7 @@
         <v>36</v>
       </c>
       <c r="G5" s="19">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>37</v>
@@ -3477,7 +3477,7 @@
         <v>36</v>
       </c>
       <c r="G6" s="19">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>37</v>
@@ -3503,7 +3503,7 @@
         <v>36</v>
       </c>
       <c r="G7" s="19">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>37</v>
@@ -3529,7 +3529,7 @@
         <v>36</v>
       </c>
       <c r="G8" s="19">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>37</v>
@@ -3555,7 +3555,7 @@
         <v>36</v>
       </c>
       <c r="G9" s="19">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>37</v>
@@ -3581,7 +3581,7 @@
         <v>36</v>
       </c>
       <c r="G10" s="19">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>37</v>
@@ -3607,7 +3607,7 @@
         <v>36</v>
       </c>
       <c r="G11" s="19">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>37</v>
@@ -3633,7 +3633,7 @@
         <v>36</v>
       </c>
       <c r="G12" s="19">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>37</v>
@@ -3659,7 +3659,7 @@
         <v>36</v>
       </c>
       <c r="G13" s="19">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>37</v>
@@ -3685,7 +3685,7 @@
         <v>36</v>
       </c>
       <c r="G14" s="19">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>37</v>
@@ -3711,7 +3711,7 @@
         <v>36</v>
       </c>
       <c r="G15" s="19">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="H15" s="17" t="s">
         <v>37</v>
@@ -3737,7 +3737,7 @@
         <v>36</v>
       </c>
       <c r="G16" s="19">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>37</v>
@@ -3763,7 +3763,7 @@
         <v>36</v>
       </c>
       <c r="G17" s="19">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H17" s="17" t="s">
         <v>37</v>
@@ -3789,7 +3789,7 @@
         <v>36</v>
       </c>
       <c r="G18" s="19">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>37</v>
@@ -3815,7 +3815,7 @@
         <v>36</v>
       </c>
       <c r="G19" s="19">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H19" s="17" t="s">
         <v>37</v>
@@ -3841,7 +3841,7 @@
         <v>36</v>
       </c>
       <c r="G20" s="19">
-        <v>36</v>
+        <v>24</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>37</v>
@@ -3867,7 +3867,7 @@
         <v>36</v>
       </c>
       <c r="G21" s="19">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="H21" s="17" t="s">
         <v>37</v>
@@ -3893,7 +3893,7 @@
         <v>36</v>
       </c>
       <c r="G22" s="19">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>37</v>
@@ -3919,7 +3919,7 @@
         <v>36</v>
       </c>
       <c r="G23" s="19">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="H23" s="17" t="s">
         <v>37</v>
@@ -3945,7 +3945,7 @@
         <v>36</v>
       </c>
       <c r="G24" s="19">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="H24" s="17" t="s">
         <v>37</v>
@@ -3971,7 +3971,7 @@
         <v>36</v>
       </c>
       <c r="G25" s="19">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>37</v>
@@ -3997,7 +3997,7 @@
         <v>36</v>
       </c>
       <c r="G26" s="19">
-        <v>1</v>
+        <v>34</v>
       </c>
       <c r="H26" s="17" t="s">
         <v>37</v>
@@ -4023,7 +4023,7 @@
         <v>36</v>
       </c>
       <c r="G27" s="19">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H27" s="17" t="s">
         <v>37</v>
@@ -4049,7 +4049,7 @@
         <v>36</v>
       </c>
       <c r="G28" s="19">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H28" s="17" t="s">
         <v>37</v>
@@ -4075,7 +4075,7 @@
         <v>36</v>
       </c>
       <c r="G29" s="19">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H29" s="17" t="s">
         <v>37</v>
@@ -4101,7 +4101,7 @@
         <v>36</v>
       </c>
       <c r="G30" s="19">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>37</v>
@@ -4127,7 +4127,7 @@
         <v>36</v>
       </c>
       <c r="G31" s="19">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="H31" s="17" t="s">
         <v>37</v>
@@ -4153,7 +4153,7 @@
         <v>36</v>
       </c>
       <c r="G32" s="19">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>37</v>
@@ -4179,7 +4179,7 @@
         <v>36</v>
       </c>
       <c r="G33" s="19">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H33" s="17" t="s">
         <v>37</v>
@@ -4205,7 +4205,7 @@
         <v>36</v>
       </c>
       <c r="G34" s="19">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H34" s="17" t="s">
         <v>37</v>
@@ -4231,7 +4231,7 @@
         <v>36</v>
       </c>
       <c r="G35" s="19">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H35" s="17" t="s">
         <v>37</v>
@@ -4257,7 +4257,7 @@
         <v>36</v>
       </c>
       <c r="G36" s="19">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="H36" s="17" t="s">
         <v>37</v>
@@ -4283,7 +4283,7 @@
         <v>36</v>
       </c>
       <c r="G37" s="19">
-        <v>9</v>
+        <v>39</v>
       </c>
       <c r="H37" s="17" t="s">
         <v>37</v>
@@ -4309,7 +4309,7 @@
         <v>36</v>
       </c>
       <c r="G38" s="19">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="H38" s="17" t="s">
         <v>37</v>
@@ -4335,7 +4335,7 @@
         <v>36</v>
       </c>
       <c r="G39" s="19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H39" s="17" t="s">
         <v>37</v>
@@ -4361,7 +4361,7 @@
         <v>36</v>
       </c>
       <c r="G40" s="19">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="H40" s="17" t="s">
         <v>37</v>
@@ -4387,7 +4387,7 @@
         <v>36</v>
       </c>
       <c r="G41" s="19">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="H41" s="17" t="s">
         <v>37</v>
@@ -4413,7 +4413,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="19">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>37</v>
@@ -4439,7 +4439,7 @@
         <v>36</v>
       </c>
       <c r="G43" s="19">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H43" s="17" t="s">
         <v>37</v>
@@ -4465,7 +4465,7 @@
         <v>36</v>
       </c>
       <c r="G44" s="19">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H44" s="17" t="s">
         <v>37</v>
@@ -4491,7 +4491,7 @@
         <v>36</v>
       </c>
       <c r="G45" s="19">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="H45" s="17" t="s">
         <v>37</v>
@@ -4543,7 +4543,7 @@
         <v>36</v>
       </c>
       <c r="G47" s="19">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H47" s="17" t="s">
         <v>37</v>
@@ -4569,7 +4569,7 @@
         <v>36</v>
       </c>
       <c r="G48" s="19">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="H48" s="17" t="s">
         <v>37</v>
@@ -4595,7 +4595,7 @@
         <v>36</v>
       </c>
       <c r="G49" s="19">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="H49" s="17" t="s">
         <v>37</v>
@@ -4621,7 +4621,7 @@
         <v>36</v>
       </c>
       <c r="G50" s="19">
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="H50" s="17" t="s">
         <v>37</v>
@@ -4647,7 +4647,7 @@
         <v>36</v>
       </c>
       <c r="G51" s="19">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="H51" s="17" t="s">
         <v>37</v>
@@ -4673,7 +4673,7 @@
         <v>36</v>
       </c>
       <c r="G52" s="19">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H52" s="17" t="s">
         <v>37</v>
@@ -4699,7 +4699,7 @@
         <v>36</v>
       </c>
       <c r="G53" s="19">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="H53" s="17" t="s">
         <v>37</v>
@@ -4725,7 +4725,7 @@
         <v>36</v>
       </c>
       <c r="G54" s="19">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="H54" s="17" t="s">
         <v>37</v>
@@ -4751,7 +4751,7 @@
         <v>36</v>
       </c>
       <c r="G55" s="19">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="H55" s="17" t="s">
         <v>37</v>
@@ -4777,7 +4777,7 @@
         <v>36</v>
       </c>
       <c r="G56" s="19">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="H56" s="17" t="s">
         <v>37</v>
@@ -4803,7 +4803,7 @@
         <v>36</v>
       </c>
       <c r="G57" s="19">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H57" s="17" t="s">
         <v>37</v>
@@ -4829,7 +4829,7 @@
         <v>36</v>
       </c>
       <c r="G58" s="19">
-        <v>30</v>
+        <v>14</v>
       </c>
       <c r="H58" s="17" t="s">
         <v>37</v>
@@ -4855,7 +4855,7 @@
         <v>36</v>
       </c>
       <c r="G59" s="19">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="H59" s="17" t="s">
         <v>37</v>
@@ -4881,7 +4881,7 @@
         <v>36</v>
       </c>
       <c r="G60" s="19">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="H60" s="17" t="s">
         <v>37</v>
@@ -4907,7 +4907,7 @@
         <v>36</v>
       </c>
       <c r="G61" s="19">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="H61" s="17" t="s">
         <v>37</v>
@@ -4933,7 +4933,7 @@
         <v>36</v>
       </c>
       <c r="G62" s="19">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H62" s="17" t="s">
         <v>37</v>
@@ -4959,7 +4959,7 @@
         <v>36</v>
       </c>
       <c r="G63" s="19">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="H63" s="17" t="s">
         <v>37</v>
@@ -4985,7 +4985,7 @@
         <v>36</v>
       </c>
       <c r="G64" s="19">
-        <v>4</v>
+        <v>28</v>
       </c>
       <c r="H64" s="17" t="s">
         <v>37</v>
@@ -5011,7 +5011,7 @@
         <v>36</v>
       </c>
       <c r="G65" s="19">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="H65" s="17" t="s">
         <v>37</v>
@@ -5037,7 +5037,7 @@
         <v>36</v>
       </c>
       <c r="G66" s="19">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="H66" s="17" t="s">
         <v>37</v>
@@ -5063,7 +5063,7 @@
         <v>36</v>
       </c>
       <c r="G67" s="19">
-        <v>13</v>
+        <v>2</v>
       </c>
       <c r="H67" s="17" t="s">
         <v>37</v>
@@ -5089,7 +5089,7 @@
         <v>36</v>
       </c>
       <c r="G68" s="19">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="H68" s="17" t="s">
         <v>37</v>
@@ -5115,7 +5115,7 @@
         <v>36</v>
       </c>
       <c r="G69" s="19">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H69" s="17" t="s">
         <v>37</v>
@@ -5141,7 +5141,7 @@
         <v>36</v>
       </c>
       <c r="G70" s="19">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H70" s="17" t="s">
         <v>37</v>
@@ -5167,7 +5167,7 @@
         <v>36</v>
       </c>
       <c r="G71" s="19">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H71" s="17" t="s">
         <v>37</v>
@@ -5193,7 +5193,7 @@
         <v>36</v>
       </c>
       <c r="G72" s="19">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="H72" s="17" t="s">
         <v>37</v>
@@ -5219,7 +5219,7 @@
         <v>36</v>
       </c>
       <c r="G73" s="19">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="H73" s="17" t="s">
         <v>37</v>
@@ -5245,7 +5245,7 @@
         <v>36</v>
       </c>
       <c r="G74" s="19">
-        <v>12</v>
+        <v>31</v>
       </c>
       <c r="H74" s="17" t="s">
         <v>37</v>
@@ -5271,7 +5271,7 @@
         <v>36</v>
       </c>
       <c r="G75" s="19">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H75" s="17" t="s">
         <v>37</v>
@@ -5297,7 +5297,7 @@
         <v>36</v>
       </c>
       <c r="G76" s="19">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H76" s="17" t="s">
         <v>37</v>
@@ -5323,7 +5323,7 @@
         <v>36</v>
       </c>
       <c r="G77" s="19">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="H77" s="17" t="s">
         <v>37</v>
@@ -5349,7 +5349,7 @@
         <v>36</v>
       </c>
       <c r="G78" s="19">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="H78" s="17" t="s">
         <v>37</v>
@@ -5375,7 +5375,7 @@
         <v>36</v>
       </c>
       <c r="G79" s="19">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H79" s="17" t="s">
         <v>37</v>
@@ -5401,7 +5401,7 @@
         <v>36</v>
       </c>
       <c r="G80" s="19">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="H80" s="17" t="s">
         <v>37</v>
@@ -5427,7 +5427,7 @@
         <v>36</v>
       </c>
       <c r="G81" s="19">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H81" s="17" t="s">
         <v>37</v>
@@ -5453,7 +5453,7 @@
         <v>36</v>
       </c>
       <c r="G82" s="19">
-        <v>38</v>
+        <v>10</v>
       </c>
       <c r="H82" s="17" t="s">
         <v>37</v>
@@ -5479,7 +5479,7 @@
         <v>36</v>
       </c>
       <c r="G83" s="19">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="H83" s="17" t="s">
         <v>37</v>
@@ -5505,7 +5505,7 @@
         <v>36</v>
       </c>
       <c r="G84" s="19">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="H84" s="17" t="s">
         <v>37</v>
@@ -5531,7 +5531,7 @@
         <v>36</v>
       </c>
       <c r="G85" s="19">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="H85" s="17" t="s">
         <v>37</v>
@@ -5557,7 +5557,7 @@
         <v>36</v>
       </c>
       <c r="G86" s="19">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="H86" s="17" t="s">
         <v>37</v>
@@ -5583,7 +5583,7 @@
         <v>36</v>
       </c>
       <c r="G87" s="19">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H87" s="17" t="s">
         <v>37</v>
@@ -5635,7 +5635,7 @@
         <v>36</v>
       </c>
       <c r="G89" s="19">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="H89" s="17" t="s">
         <v>37</v>
@@ -5661,7 +5661,7 @@
         <v>36</v>
       </c>
       <c r="G90" s="19">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H90" s="17" t="s">
         <v>37</v>
@@ -5687,7 +5687,7 @@
         <v>36</v>
       </c>
       <c r="G91" s="19">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H91" s="17" t="s">
         <v>37</v>
@@ -5713,7 +5713,7 @@
         <v>36</v>
       </c>
       <c r="G92" s="19">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H92" s="17" t="s">
         <v>37</v>
@@ -5739,7 +5739,7 @@
         <v>36</v>
       </c>
       <c r="G93" s="19">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="H93" s="17" t="s">
         <v>37</v>
@@ -5765,7 +5765,7 @@
         <v>36</v>
       </c>
       <c r="G94" s="19">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="H94" s="17" t="s">
         <v>37</v>
@@ -5791,7 +5791,7 @@
         <v>36</v>
       </c>
       <c r="G95" s="19">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H95" s="17" t="s">
         <v>37</v>
@@ -5817,7 +5817,7 @@
         <v>36</v>
       </c>
       <c r="G96" s="19">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H96" s="17" t="s">
         <v>37</v>
@@ -5843,7 +5843,7 @@
         <v>36</v>
       </c>
       <c r="G97" s="19">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="H97" s="17" t="s">
         <v>37</v>
@@ -5869,7 +5869,7 @@
         <v>36</v>
       </c>
       <c r="G98" s="19">
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="H98" s="17" t="s">
         <v>37</v>
@@ -5895,7 +5895,7 @@
         <v>36</v>
       </c>
       <c r="G99" s="19">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="H99" s="17" t="s">
         <v>37</v>
@@ -5921,7 +5921,7 @@
         <v>36</v>
       </c>
       <c r="G100" s="19">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="H100" s="17" t="s">
         <v>37</v>
@@ -5947,7 +5947,7 @@
         <v>36</v>
       </c>
       <c r="G101" s="19">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H101" s="17" t="s">
         <v>37</v>
@@ -5973,7 +5973,7 @@
         <v>36</v>
       </c>
       <c r="G102" s="19">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H102" s="17" t="s">
         <v>37</v>
@@ -5999,7 +5999,7 @@
         <v>36</v>
       </c>
       <c r="G103" s="19">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="H103" s="17" t="s">
         <v>37</v>
@@ -6025,7 +6025,7 @@
         <v>36</v>
       </c>
       <c r="G104" s="19">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="H104" s="17" t="s">
         <v>37</v>
@@ -6051,7 +6051,7 @@
         <v>36</v>
       </c>
       <c r="G105" s="19">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="H105" s="17" t="s">
         <v>37</v>
@@ -6077,7 +6077,7 @@
         <v>36</v>
       </c>
       <c r="G106" s="19">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="H106" s="17" t="s">
         <v>37</v>
@@ -6103,7 +6103,7 @@
         <v>36</v>
       </c>
       <c r="G107" s="19">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="H107" s="17" t="s">
         <v>37</v>
@@ -6129,7 +6129,7 @@
         <v>36</v>
       </c>
       <c r="G108" s="19">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H108" s="17" t="s">
         <v>37</v>
@@ -6181,7 +6181,7 @@
         <v>36</v>
       </c>
       <c r="G110" s="19">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H110" s="17" t="s">
         <v>37</v>
@@ -6207,7 +6207,7 @@
         <v>36</v>
       </c>
       <c r="G111" s="19">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="H111" s="17" t="s">
         <v>37</v>
@@ -6233,7 +6233,7 @@
         <v>36</v>
       </c>
       <c r="G112" s="19">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H112" s="17" t="s">
         <v>37</v>
@@ -6259,7 +6259,7 @@
         <v>36</v>
       </c>
       <c r="G113" s="19">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="H113" s="17" t="s">
         <v>37</v>
@@ -6285,7 +6285,7 @@
         <v>36</v>
       </c>
       <c r="G114" s="19">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="H114" s="17" t="s">
         <v>37</v>
@@ -6311,7 +6311,7 @@
         <v>36</v>
       </c>
       <c r="G115" s="19">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="H115" s="17" t="s">
         <v>37</v>
@@ -6337,7 +6337,7 @@
         <v>36</v>
       </c>
       <c r="G116" s="19">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H116" s="17" t="s">
         <v>37</v>
@@ -6363,7 +6363,7 @@
         <v>36</v>
       </c>
       <c r="G117" s="19">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="H117" s="17" t="s">
         <v>37</v>
@@ -6389,7 +6389,7 @@
         <v>36</v>
       </c>
       <c r="G118" s="19">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="H118" s="17" t="s">
         <v>37</v>
@@ -6415,7 +6415,7 @@
         <v>36</v>
       </c>
       <c r="G119" s="19">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="H119" s="17" t="s">
         <v>37</v>
@@ -6441,7 +6441,7 @@
         <v>36</v>
       </c>
       <c r="G120" s="19">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H120" s="17" t="s">
         <v>37</v>
@@ -6467,7 +6467,7 @@
         <v>36</v>
       </c>
       <c r="G121" s="19">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H121" s="17" t="s">
         <v>37</v>
@@ -6493,7 +6493,7 @@
         <v>36</v>
       </c>
       <c r="G122" s="19">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="H122" s="17" t="s">
         <v>37</v>
@@ -6519,7 +6519,7 @@
         <v>36</v>
       </c>
       <c r="G123" s="19">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="H123" s="17" t="s">
         <v>37</v>
@@ -6545,7 +6545,7 @@
         <v>36</v>
       </c>
       <c r="G124" s="19">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H124" s="17" t="s">
         <v>37</v>
@@ -6571,7 +6571,7 @@
         <v>36</v>
       </c>
       <c r="G125" s="19">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="H125" s="17" t="s">
         <v>37</v>
@@ -6597,7 +6597,7 @@
         <v>36</v>
       </c>
       <c r="G126" s="19">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="H126" s="17" t="s">
         <v>37</v>
@@ -6623,7 +6623,7 @@
         <v>36</v>
       </c>
       <c r="G127" s="19">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="H127" s="17" t="s">
         <v>37</v>
@@ -6649,7 +6649,7 @@
         <v>36</v>
       </c>
       <c r="G128" s="19">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="H128" s="17" t="s">
         <v>37</v>
@@ -6675,7 +6675,7 @@
         <v>36</v>
       </c>
       <c r="G129" s="19">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="H129" s="17" t="s">
         <v>37</v>
@@ -6701,7 +6701,7 @@
         <v>36</v>
       </c>
       <c r="G130" s="19">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="H130" s="17" t="s">
         <v>37</v>
@@ -6727,7 +6727,7 @@
         <v>36</v>
       </c>
       <c r="G131" s="19">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H131" s="17" t="s">
         <v>37</v>
@@ -6753,7 +6753,7 @@
         <v>36</v>
       </c>
       <c r="G132" s="19">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="H132" s="17" t="s">
         <v>37</v>
@@ -6779,7 +6779,7 @@
         <v>36</v>
       </c>
       <c r="G133" s="19">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="H133" s="17" t="s">
         <v>37</v>
@@ -6805,7 +6805,7 @@
         <v>36</v>
       </c>
       <c r="G134" s="19">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="H134" s="17" t="s">
         <v>37</v>
@@ -6831,7 +6831,7 @@
         <v>36</v>
       </c>
       <c r="G135" s="19">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="H135" s="17" t="s">
         <v>37</v>
@@ -6857,7 +6857,7 @@
         <v>36</v>
       </c>
       <c r="G136" s="19">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="H136" s="17" t="s">
         <v>37</v>
@@ -6883,7 +6883,7 @@
         <v>36</v>
       </c>
       <c r="G137" s="19">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="H137" s="17" t="s">
         <v>37</v>
@@ -6909,7 +6909,7 @@
         <v>36</v>
       </c>
       <c r="G138" s="19">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H138" s="17" t="s">
         <v>37</v>
@@ -6935,7 +6935,7 @@
         <v>36</v>
       </c>
       <c r="G139" s="19">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="H139" s="17" t="s">
         <v>37</v>
@@ -6961,7 +6961,7 @@
         <v>36</v>
       </c>
       <c r="G140" s="19">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="H140" s="17" t="s">
         <v>37</v>
@@ -6987,7 +6987,7 @@
         <v>36</v>
       </c>
       <c r="G141" s="19">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H141" s="17" t="s">
         <v>37</v>
@@ -7013,7 +7013,7 @@
         <v>36</v>
       </c>
       <c r="G142" s="19">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="H142" s="17" t="s">
         <v>37</v>
@@ -7065,7 +7065,7 @@
         <v>36</v>
       </c>
       <c r="G144" s="19">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H144" s="17" t="s">
         <v>37</v>
@@ -7091,7 +7091,7 @@
         <v>36</v>
       </c>
       <c r="G145" s="19">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H145" s="17" t="s">
         <v>37</v>
@@ -7117,7 +7117,7 @@
         <v>36</v>
       </c>
       <c r="G146" s="19">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="H146" s="17" t="s">
         <v>37</v>
@@ -7143,7 +7143,7 @@
         <v>36</v>
       </c>
       <c r="G147" s="19">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H147" s="17" t="s">
         <v>37</v>
@@ -7169,7 +7169,7 @@
         <v>36</v>
       </c>
       <c r="G148" s="19">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H148" s="17" t="s">
         <v>37</v>
@@ -7195,7 +7195,7 @@
         <v>36</v>
       </c>
       <c r="G149" s="19">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="H149" s="17" t="s">
         <v>37</v>
@@ -7221,7 +7221,7 @@
         <v>36</v>
       </c>
       <c r="G150" s="19">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="H150" s="17" t="s">
         <v>37</v>
@@ -7247,7 +7247,7 @@
         <v>36</v>
       </c>
       <c r="G151" s="19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H151" s="17" t="s">
         <v>37</v>
@@ -7273,7 +7273,7 @@
         <v>36</v>
       </c>
       <c r="G152" s="19">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="H152" s="17" t="s">
         <v>37</v>
@@ -7299,7 +7299,7 @@
         <v>36</v>
       </c>
       <c r="G153" s="19">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H153" s="17" t="s">
         <v>37</v>
@@ -7325,7 +7325,7 @@
         <v>36</v>
       </c>
       <c r="G154" s="19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H154" s="17" t="s">
         <v>37</v>
@@ -7351,7 +7351,7 @@
         <v>36</v>
       </c>
       <c r="G155" s="19">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H155" s="17" t="s">
         <v>37</v>
@@ -7377,7 +7377,7 @@
         <v>36</v>
       </c>
       <c r="G156" s="19">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="H156" s="17" t="s">
         <v>37</v>
@@ -7403,7 +7403,7 @@
         <v>36</v>
       </c>
       <c r="G157" s="19">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="H157" s="17" t="s">
         <v>37</v>
@@ -7429,7 +7429,7 @@
         <v>36</v>
       </c>
       <c r="G158" s="19">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H158" s="17" t="s">
         <v>37</v>
@@ -7455,7 +7455,7 @@
         <v>36</v>
       </c>
       <c r="G159" s="19">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="H159" s="17" t="s">
         <v>37</v>
@@ -7481,7 +7481,7 @@
         <v>36</v>
       </c>
       <c r="G160" s="19">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="H160" s="17" t="s">
         <v>37</v>
@@ -7507,7 +7507,7 @@
         <v>36</v>
       </c>
       <c r="G161" s="19">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H161" s="17" t="s">
         <v>37</v>
@@ -7533,7 +7533,7 @@
         <v>36</v>
       </c>
       <c r="G162" s="19">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="H162" s="17" t="s">
         <v>37</v>
@@ -7559,7 +7559,7 @@
         <v>36</v>
       </c>
       <c r="G163" s="19">
-        <v>37</v>
+        <v>9</v>
       </c>
       <c r="H163" s="17" t="s">
         <v>37</v>
@@ -7585,7 +7585,7 @@
         <v>36</v>
       </c>
       <c r="G164" s="19">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="H164" s="17" t="s">
         <v>37</v>
@@ -7611,7 +7611,7 @@
         <v>36</v>
       </c>
       <c r="G165" s="19">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H165" s="17" t="s">
         <v>37</v>
@@ -7637,7 +7637,7 @@
         <v>36</v>
       </c>
       <c r="G166" s="19">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H166" s="17" t="s">
         <v>37</v>
@@ -7663,7 +7663,7 @@
         <v>36</v>
       </c>
       <c r="G167" s="19">
-        <v>15</v>
+        <v>35</v>
       </c>
       <c r="H167" s="17" t="s">
         <v>37</v>
@@ -7715,7 +7715,7 @@
         <v>36</v>
       </c>
       <c r="G169" s="19">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H169" s="17" t="s">
         <v>37</v>
@@ -7741,7 +7741,7 @@
         <v>36</v>
       </c>
       <c r="G170" s="19">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H170" s="17" t="s">
         <v>37</v>
@@ -7767,7 +7767,7 @@
         <v>36</v>
       </c>
       <c r="G171" s="19">
-        <v>37</v>
+        <v>12</v>
       </c>
       <c r="H171" s="17" t="s">
         <v>37</v>
@@ -7793,7 +7793,7 @@
         <v>36</v>
       </c>
       <c r="G172" s="19">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="H172" s="17" t="s">
         <v>37</v>
@@ -7819,7 +7819,7 @@
         <v>36</v>
       </c>
       <c r="G173" s="19">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H173" s="17" t="s">
         <v>37</v>
@@ -7845,7 +7845,7 @@
         <v>36</v>
       </c>
       <c r="G174" s="19">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="H174" s="17" t="s">
         <v>37</v>
@@ -7871,7 +7871,7 @@
         <v>36</v>
       </c>
       <c r="G175" s="19">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="H175" s="17" t="s">
         <v>37</v>
@@ -7897,7 +7897,7 @@
         <v>36</v>
       </c>
       <c r="G176" s="19">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H176" s="17" t="s">
         <v>37</v>
@@ -7923,7 +7923,7 @@
         <v>36</v>
       </c>
       <c r="G177" s="19">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H177" s="17" t="s">
         <v>37</v>
@@ -7949,7 +7949,7 @@
         <v>36</v>
       </c>
       <c r="G178" s="19">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="H178" s="17" t="s">
         <v>37</v>
@@ -7975,7 +7975,7 @@
         <v>36</v>
       </c>
       <c r="G179" s="19">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="H179" s="17" t="s">
         <v>37</v>
@@ -8001,7 +8001,7 @@
         <v>36</v>
       </c>
       <c r="G180" s="19">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H180" s="17" t="s">
         <v>37</v>
@@ -8027,7 +8027,7 @@
         <v>36</v>
       </c>
       <c r="G181" s="19">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="H181" s="17" t="s">
         <v>37</v>
@@ -8053,7 +8053,7 @@
         <v>36</v>
       </c>
       <c r="G182" s="19">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H182" s="17" t="s">
         <v>37</v>
@@ -8079,7 +8079,7 @@
         <v>36</v>
       </c>
       <c r="G183" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H183" s="17" t="s">
         <v>37</v>
@@ -8105,7 +8105,7 @@
         <v>36</v>
       </c>
       <c r="G184" s="19">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H184" s="17" t="s">
         <v>37</v>
@@ -8131,7 +8131,7 @@
         <v>36</v>
       </c>
       <c r="G185" s="19">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="H185" s="17" t="s">
         <v>37</v>
@@ -8157,7 +8157,7 @@
         <v>36</v>
       </c>
       <c r="G186" s="19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H186" s="17" t="s">
         <v>37</v>
@@ -8183,7 +8183,7 @@
         <v>36</v>
       </c>
       <c r="G187" s="19">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="H187" s="17" t="s">
         <v>37</v>
@@ -8209,7 +8209,7 @@
         <v>36</v>
       </c>
       <c r="G188" s="19">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="H188" s="17" t="s">
         <v>37</v>
@@ -8235,7 +8235,7 @@
         <v>36</v>
       </c>
       <c r="G189" s="19">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="H189" s="17" t="s">
         <v>37</v>
@@ -8261,7 +8261,7 @@
         <v>36</v>
       </c>
       <c r="G190" s="19">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="H190" s="17" t="s">
         <v>37</v>
@@ -8287,7 +8287,7 @@
         <v>36</v>
       </c>
       <c r="G191" s="19">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="H191" s="17" t="s">
         <v>37</v>
@@ -8313,7 +8313,7 @@
         <v>36</v>
       </c>
       <c r="G192" s="19">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="H192" s="17" t="s">
         <v>37</v>
@@ -8339,7 +8339,7 @@
         <v>36</v>
       </c>
       <c r="G193" s="19">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="H193" s="17" t="s">
         <v>37</v>
@@ -8365,7 +8365,7 @@
         <v>36</v>
       </c>
       <c r="G194" s="19">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H194" s="17" t="s">
         <v>37</v>
@@ -8391,7 +8391,7 @@
         <v>36</v>
       </c>
       <c r="G195" s="19">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="H195" s="17" t="s">
         <v>37</v>
@@ -8417,7 +8417,7 @@
         <v>36</v>
       </c>
       <c r="G196" s="19">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="H196" s="17" t="s">
         <v>37</v>
@@ -8443,7 +8443,7 @@
         <v>36</v>
       </c>
       <c r="G197" s="19">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="H197" s="17" t="s">
         <v>37</v>
@@ -8469,7 +8469,7 @@
         <v>36</v>
       </c>
       <c r="G198" s="19">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="H198" s="17" t="s">
         <v>37</v>
@@ -8495,7 +8495,7 @@
         <v>36</v>
       </c>
       <c r="G199" s="19">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="H199" s="17" t="s">
         <v>37</v>
@@ -8521,7 +8521,7 @@
         <v>36</v>
       </c>
       <c r="G200" s="19">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H200" s="17" t="s">
         <v>37</v>
@@ -8547,7 +8547,7 @@
         <v>36</v>
       </c>
       <c r="G201" s="19">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H201" s="17" t="s">
         <v>37</v>
@@ -8573,7 +8573,7 @@
         <v>36</v>
       </c>
       <c r="G202" s="19">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="H202" s="17" t="s">
         <v>37</v>
@@ -8599,7 +8599,7 @@
         <v>36</v>
       </c>
       <c r="G203" s="19">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="H203" s="17" t="s">
         <v>37</v>
@@ -8625,7 +8625,7 @@
         <v>36</v>
       </c>
       <c r="G204" s="19">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="H204" s="17" t="s">
         <v>37</v>
@@ -8651,7 +8651,7 @@
         <v>36</v>
       </c>
       <c r="G205" s="19">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H205" s="17" t="s">
         <v>37</v>
@@ -8677,7 +8677,7 @@
         <v>36</v>
       </c>
       <c r="G206" s="19">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="H206" s="17" t="s">
         <v>37</v>
@@ -8703,7 +8703,7 @@
         <v>36</v>
       </c>
       <c r="G207" s="19">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="H207" s="17" t="s">
         <v>37</v>
@@ -8729,7 +8729,7 @@
         <v>36</v>
       </c>
       <c r="G208" s="19">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H208" s="17" t="s">
         <v>37</v>
@@ -8755,7 +8755,7 @@
         <v>36</v>
       </c>
       <c r="G209" s="19">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="H209" s="17" t="s">
         <v>37</v>
@@ -8781,7 +8781,7 @@
         <v>36</v>
       </c>
       <c r="G210" s="19">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="H210" s="17" t="s">
         <v>37</v>
@@ -8807,7 +8807,7 @@
         <v>36</v>
       </c>
       <c r="G211" s="19">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H211" s="17" t="s">
         <v>37</v>
@@ -8833,7 +8833,7 @@
         <v>36</v>
       </c>
       <c r="G212" s="19">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="H212" s="17" t="s">
         <v>37</v>
@@ -8859,7 +8859,7 @@
         <v>36</v>
       </c>
       <c r="G213" s="19">
-        <v>8</v>
+        <v>25</v>
       </c>
       <c r="H213" s="17" t="s">
         <v>37</v>
@@ -8885,7 +8885,7 @@
         <v>36</v>
       </c>
       <c r="G214" s="19">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="H214" s="17" t="s">
         <v>37</v>
@@ -8911,7 +8911,7 @@
         <v>36</v>
       </c>
       <c r="G215" s="19">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H215" s="17" t="s">
         <v>37</v>
@@ -8937,7 +8937,7 @@
         <v>36</v>
       </c>
       <c r="G216" s="19">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="H216" s="17" t="s">
         <v>37</v>
@@ -8963,7 +8963,7 @@
         <v>36</v>
       </c>
       <c r="G217" s="19">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="H217" s="17" t="s">
         <v>37</v>
@@ -8989,7 +8989,7 @@
         <v>36</v>
       </c>
       <c r="G218" s="19">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="H218" s="17" t="s">
         <v>37</v>
@@ -9015,7 +9015,7 @@
         <v>36</v>
       </c>
       <c r="G219" s="19">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H219" s="17" t="s">
         <v>37</v>
@@ -9041,7 +9041,7 @@
         <v>36</v>
       </c>
       <c r="G220" s="19">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="H220" s="17" t="s">
         <v>37</v>
@@ -9067,7 +9067,7 @@
         <v>36</v>
       </c>
       <c r="G221" s="19">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="H221" s="17" t="s">
         <v>37</v>
@@ -9093,7 +9093,7 @@
         <v>36</v>
       </c>
       <c r="G222" s="19">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H222" s="17" t="s">
         <v>37</v>
@@ -9119,7 +9119,7 @@
         <v>36</v>
       </c>
       <c r="G223" s="19">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H223" s="17" t="s">
         <v>37</v>
@@ -9145,7 +9145,7 @@
         <v>36</v>
       </c>
       <c r="G224" s="19">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="H224" s="17" t="s">
         <v>37</v>
@@ -9171,7 +9171,7 @@
         <v>36</v>
       </c>
       <c r="G225" s="19">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="H225" s="17" t="s">
         <v>37</v>
@@ -9197,7 +9197,7 @@
         <v>36</v>
       </c>
       <c r="G226" s="19">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H226" s="17" t="s">
         <v>37</v>
@@ -9223,7 +9223,7 @@
         <v>36</v>
       </c>
       <c r="G227" s="19">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="H227" s="17" t="s">
         <v>37</v>
@@ -9249,7 +9249,7 @@
         <v>36</v>
       </c>
       <c r="G228" s="19">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="H228" s="17" t="s">
         <v>37</v>
@@ -9275,7 +9275,7 @@
         <v>36</v>
       </c>
       <c r="G229" s="19">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H229" s="17" t="s">
         <v>37</v>
@@ -9301,7 +9301,7 @@
         <v>36</v>
       </c>
       <c r="G230" s="19">
-        <v>38</v>
+        <v>7</v>
       </c>
       <c r="H230" s="17" t="s">
         <v>37</v>
@@ -9327,7 +9327,7 @@
         <v>36</v>
       </c>
       <c r="G231" s="19">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="H231" s="17" t="s">
         <v>37</v>
@@ -9353,7 +9353,7 @@
         <v>36</v>
       </c>
       <c r="G232" s="19">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="H232" s="17" t="s">
         <v>37</v>
@@ -9379,7 +9379,7 @@
         <v>36</v>
       </c>
       <c r="G233" s="19">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H233" s="17" t="s">
         <v>37</v>
@@ -9431,7 +9431,7 @@
         <v>36</v>
       </c>
       <c r="G235" s="19">
-        <v>7</v>
+        <v>38</v>
       </c>
       <c r="H235" s="17" t="s">
         <v>37</v>
@@ -9457,7 +9457,7 @@
         <v>36</v>
       </c>
       <c r="G236" s="19">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="H236" s="17" t="s">
         <v>37</v>
@@ -9483,7 +9483,7 @@
         <v>36</v>
       </c>
       <c r="G237" s="19">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="H237" s="17" t="s">
         <v>37</v>
@@ -9509,7 +9509,7 @@
         <v>36</v>
       </c>
       <c r="G238" s="19">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="H238" s="17" t="s">
         <v>37</v>
@@ -9535,7 +9535,7 @@
         <v>36</v>
       </c>
       <c r="G239" s="19">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="H239" s="17" t="s">
         <v>37</v>
@@ -9561,7 +9561,7 @@
         <v>36</v>
       </c>
       <c r="G240" s="19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H240" s="17" t="s">
         <v>37</v>
@@ -9587,7 +9587,7 @@
         <v>36</v>
       </c>
       <c r="G241" s="19">
-        <v>28</v>
+        <v>35</v>
       </c>
       <c r="H241" s="17" t="s">
         <v>37</v>
@@ -9613,7 +9613,7 @@
         <v>36</v>
       </c>
       <c r="G242" s="19">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H242" s="17" t="s">
         <v>37</v>
@@ -9639,7 +9639,7 @@
         <v>36</v>
       </c>
       <c r="G243" s="19">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H243" s="17" t="s">
         <v>37</v>
@@ -9665,7 +9665,7 @@
         <v>36</v>
       </c>
       <c r="G244" s="19">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="H244" s="17" t="s">
         <v>37</v>
@@ -9691,7 +9691,7 @@
         <v>36</v>
       </c>
       <c r="G245" s="19">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H245" s="17" t="s">
         <v>37</v>
@@ -9717,7 +9717,7 @@
         <v>36</v>
       </c>
       <c r="G246" s="19">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H246" s="17" t="s">
         <v>37</v>
@@ -9743,7 +9743,7 @@
         <v>36</v>
       </c>
       <c r="G247" s="19">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="H247" s="17" t="s">
         <v>37</v>
@@ -9769,7 +9769,7 @@
         <v>36</v>
       </c>
       <c r="G248" s="19">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="H248" s="17" t="s">
         <v>37</v>
@@ -9795,7 +9795,7 @@
         <v>36</v>
       </c>
       <c r="G249" s="19">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="H249" s="17" t="s">
         <v>37</v>
@@ -9821,7 +9821,7 @@
         <v>36</v>
       </c>
       <c r="G250" s="19">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H250" s="17" t="s">
         <v>37</v>
@@ -9847,7 +9847,7 @@
         <v>36</v>
       </c>
       <c r="G251" s="19">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H251" s="17" t="s">
         <v>37</v>
@@ -9873,7 +9873,7 @@
         <v>36</v>
       </c>
       <c r="G252" s="19">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="H252" s="17" t="s">
         <v>37</v>
@@ -9925,7 +9925,7 @@
         <v>36</v>
       </c>
       <c r="G254" s="19">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H254" s="17" t="s">
         <v>37</v>
@@ -9951,7 +9951,7 @@
         <v>36</v>
       </c>
       <c r="G255" s="19">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="H255" s="17" t="s">
         <v>37</v>
@@ -9977,7 +9977,7 @@
         <v>36</v>
       </c>
       <c r="G256" s="19">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H256" s="17" t="s">
         <v>37</v>
@@ -10003,7 +10003,7 @@
         <v>36</v>
       </c>
       <c r="G257" s="19">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="H257" s="17" t="s">
         <v>37</v>
@@ -10029,7 +10029,7 @@
         <v>36</v>
       </c>
       <c r="G258" s="19">
-        <v>35</v>
+        <v>4</v>
       </c>
       <c r="H258" s="17" t="s">
         <v>37</v>
@@ -10055,7 +10055,7 @@
         <v>36</v>
       </c>
       <c r="G259" s="19">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="H259" s="17" t="s">
         <v>37</v>
@@ -10081,7 +10081,7 @@
         <v>36</v>
       </c>
       <c r="G260" s="19">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="H260" s="17" t="s">
         <v>37</v>
@@ -10107,7 +10107,7 @@
         <v>36</v>
       </c>
       <c r="G261" s="19">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="H261" s="17" t="s">
         <v>37</v>
@@ -10133,7 +10133,7 @@
         <v>36</v>
       </c>
       <c r="G262" s="19">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="H262" s="17" t="s">
         <v>37</v>
@@ -10159,7 +10159,7 @@
         <v>36</v>
       </c>
       <c r="G263" s="19">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H263" s="17" t="s">
         <v>37</v>
@@ -10185,7 +10185,7 @@
         <v>36</v>
       </c>
       <c r="G264" s="19">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="H264" s="17" t="s">
         <v>37</v>
@@ -10211,7 +10211,7 @@
         <v>36</v>
       </c>
       <c r="G265" s="19">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="H265" s="17" t="s">
         <v>37</v>
@@ -10237,7 +10237,7 @@
         <v>36</v>
       </c>
       <c r="G266" s="19">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="H266" s="17" t="s">
         <v>37</v>
@@ -10263,7 +10263,7 @@
         <v>36</v>
       </c>
       <c r="G267" s="19">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="H267" s="17" t="s">
         <v>37</v>
@@ -10289,7 +10289,7 @@
         <v>36</v>
       </c>
       <c r="G268" s="19">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="H268" s="17" t="s">
         <v>37</v>
@@ -10315,7 +10315,7 @@
         <v>36</v>
       </c>
       <c r="G269" s="19">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H269" s="17" t="s">
         <v>37</v>
@@ -10341,7 +10341,7 @@
         <v>36</v>
       </c>
       <c r="G270" s="19">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H270" s="17" t="s">
         <v>37</v>
@@ -10367,7 +10367,7 @@
         <v>36</v>
       </c>
       <c r="G271" s="19">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="H271" s="17" t="s">
         <v>37</v>
@@ -10393,7 +10393,7 @@
         <v>36</v>
       </c>
       <c r="G272" s="19">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="H272" s="17" t="s">
         <v>37</v>
@@ -10419,7 +10419,7 @@
         <v>36</v>
       </c>
       <c r="G273" s="19">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="H273" s="17" t="s">
         <v>37</v>
@@ -10445,7 +10445,7 @@
         <v>36</v>
       </c>
       <c r="G274" s="19">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="H274" s="17" t="s">
         <v>37</v>
@@ -10471,7 +10471,7 @@
         <v>36</v>
       </c>
       <c r="G275" s="19">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="H275" s="17" t="s">
         <v>37</v>
@@ -10497,7 +10497,7 @@
         <v>36</v>
       </c>
       <c r="G276" s="19">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="H276" s="17" t="s">
         <v>37</v>
@@ -10523,7 +10523,7 @@
         <v>36</v>
       </c>
       <c r="G277" s="19">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="H277" s="17" t="s">
         <v>37</v>
@@ -10549,7 +10549,7 @@
         <v>36</v>
       </c>
       <c r="G278" s="19">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="H278" s="17" t="s">
         <v>37</v>
@@ -10575,7 +10575,7 @@
         <v>36</v>
       </c>
       <c r="G279" s="19">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H279" s="17" t="s">
         <v>37</v>
@@ -10601,7 +10601,7 @@
         <v>36</v>
       </c>
       <c r="G280" s="19">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="H280" s="17" t="s">
         <v>37</v>
@@ -10627,7 +10627,7 @@
         <v>36</v>
       </c>
       <c r="G281" s="19">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H281" s="17" t="s">
         <v>37</v>
@@ -10679,7 +10679,7 @@
         <v>36</v>
       </c>
       <c r="G283" s="19">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H283" s="17" t="s">
         <v>37</v>
@@ -10705,7 +10705,7 @@
         <v>36</v>
       </c>
       <c r="G284" s="19">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H284" s="17" t="s">
         <v>37</v>
@@ -10731,7 +10731,7 @@
         <v>36</v>
       </c>
       <c r="G285" s="19">
-        <v>28</v>
+        <v>6</v>
       </c>
       <c r="H285" s="17" t="s">
         <v>37</v>
@@ -10757,7 +10757,7 @@
         <v>36</v>
       </c>
       <c r="G286" s="19">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H286" s="17" t="s">
         <v>37</v>
@@ -10783,7 +10783,7 @@
         <v>36</v>
       </c>
       <c r="G287" s="19">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="H287" s="17" t="s">
         <v>37</v>
@@ -10809,7 +10809,7 @@
         <v>36</v>
       </c>
       <c r="G288" s="19">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="H288" s="17" t="s">
         <v>37</v>
@@ -10835,7 +10835,7 @@
         <v>36</v>
       </c>
       <c r="G289" s="19">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="H289" s="17" t="s">
         <v>37</v>
@@ -10861,7 +10861,7 @@
         <v>36</v>
       </c>
       <c r="G290" s="19">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="H290" s="17" t="s">
         <v>37</v>
@@ -10887,7 +10887,7 @@
         <v>36</v>
       </c>
       <c r="G291" s="19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H291" s="17" t="s">
         <v>37</v>
@@ -10913,7 +10913,7 @@
         <v>36</v>
       </c>
       <c r="G292" s="19">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="H292" s="17" t="s">
         <v>37</v>
@@ -10965,7 +10965,7 @@
         <v>36</v>
       </c>
       <c r="G294" s="19">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H294" s="17" t="s">
         <v>37</v>
@@ -10991,7 +10991,7 @@
         <v>36</v>
       </c>
       <c r="G295" s="19">
-        <v>39</v>
+        <v>2</v>
       </c>
       <c r="H295" s="17" t="s">
         <v>37</v>
@@ -11017,7 +11017,7 @@
         <v>36</v>
       </c>
       <c r="G296" s="19">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="H296" s="17" t="s">
         <v>37</v>
@@ -11043,7 +11043,7 @@
         <v>36</v>
       </c>
       <c r="G297" s="19">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="H297" s="17" t="s">
         <v>37</v>
@@ -11069,7 +11069,7 @@
         <v>36</v>
       </c>
       <c r="G298" s="19">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="H298" s="17" t="s">
         <v>37</v>
@@ -11095,7 +11095,7 @@
         <v>36</v>
       </c>
       <c r="G299" s="19">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="H299" s="17" t="s">
         <v>37</v>
@@ -11121,7 +11121,7 @@
         <v>36</v>
       </c>
       <c r="G300" s="19">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="H300" s="17" t="s">
         <v>37</v>
@@ -11147,7 +11147,7 @@
         <v>36</v>
       </c>
       <c r="G301" s="19">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="H301" s="17" t="s">
         <v>37</v>
@@ -11173,7 +11173,7 @@
         <v>36</v>
       </c>
       <c r="G302" s="19">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="H302" s="17" t="s">
         <v>37</v>
@@ -11199,7 +11199,7 @@
         <v>36</v>
       </c>
       <c r="G303" s="19">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="H303" s="17" t="s">
         <v>37</v>
@@ -11225,7 +11225,7 @@
         <v>36</v>
       </c>
       <c r="G304" s="19">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="H304" s="17" t="s">
         <v>37</v>
@@ -11251,7 +11251,7 @@
         <v>36</v>
       </c>
       <c r="G305" s="19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="H305" s="17" t="s">
         <v>37</v>
@@ -11277,7 +11277,7 @@
         <v>36</v>
       </c>
       <c r="G306" s="19">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H306" s="17" t="s">
         <v>37</v>
@@ -11303,7 +11303,7 @@
         <v>36</v>
       </c>
       <c r="G307" s="19">
-        <v>32</v>
+        <v>15</v>
       </c>
       <c r="H307" s="17" t="s">
         <v>37</v>
@@ -11355,7 +11355,7 @@
         <v>36</v>
       </c>
       <c r="G309" s="19">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H309" s="17" t="s">
         <v>37</v>
@@ -11381,7 +11381,7 @@
         <v>36</v>
       </c>
       <c r="G310" s="19">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="H310" s="17" t="s">
         <v>37</v>
@@ -11407,7 +11407,7 @@
         <v>36</v>
       </c>
       <c r="G311" s="19">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="H311" s="17" t="s">
         <v>37</v>
@@ -11433,7 +11433,7 @@
         <v>36</v>
       </c>
       <c r="G312" s="19">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H312" s="17" t="s">
         <v>37</v>
@@ -11459,7 +11459,7 @@
         <v>36</v>
       </c>
       <c r="G313" s="19">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="H313" s="17" t="s">
         <v>37</v>
@@ -11485,7 +11485,7 @@
         <v>36</v>
       </c>
       <c r="G314" s="19">
-        <v>4</v>
+        <v>38</v>
       </c>
       <c r="H314" s="17" t="s">
         <v>37</v>
@@ -11511,7 +11511,7 @@
         <v>36</v>
       </c>
       <c r="G315" s="19">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H315" s="17" t="s">
         <v>37</v>
@@ -11537,7 +11537,7 @@
         <v>36</v>
       </c>
       <c r="G316" s="19">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="H316" s="17" t="s">
         <v>37</v>
@@ -11563,7 +11563,7 @@
         <v>36</v>
       </c>
       <c r="G317" s="19">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="H317" s="17" t="s">
         <v>37</v>
@@ -11589,7 +11589,7 @@
         <v>36</v>
       </c>
       <c r="G318" s="19">
-        <v>4</v>
+        <v>39</v>
       </c>
       <c r="H318" s="17" t="s">
         <v>37</v>
@@ -11615,7 +11615,7 @@
         <v>36</v>
       </c>
       <c r="G319" s="19">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H319" s="17" t="s">
         <v>37</v>
@@ -11641,7 +11641,7 @@
         <v>36</v>
       </c>
       <c r="G320" s="19">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H320" s="17" t="s">
         <v>37</v>
@@ -11667,7 +11667,7 @@
         <v>36</v>
       </c>
       <c r="G321" s="19">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="H321" s="17" t="s">
         <v>37</v>
@@ -11693,7 +11693,7 @@
         <v>36</v>
       </c>
       <c r="G322" s="19">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="H322" s="17" t="s">
         <v>37</v>
@@ -11719,7 +11719,7 @@
         <v>36</v>
       </c>
       <c r="G323" s="19">
-        <v>39</v>
+        <v>6</v>
       </c>
       <c r="H323" s="17" t="s">
         <v>37</v>
@@ -11745,7 +11745,7 @@
         <v>36</v>
       </c>
       <c r="G324" s="19">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H324" s="17" t="s">
         <v>37</v>
@@ -11771,7 +11771,7 @@
         <v>36</v>
       </c>
       <c r="G325" s="19">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="H325" s="17" t="s">
         <v>37</v>
@@ -11797,7 +11797,7 @@
         <v>36</v>
       </c>
       <c r="G326" s="19">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="H326" s="17" t="s">
         <v>37</v>
@@ -11823,7 +11823,7 @@
         <v>36</v>
       </c>
       <c r="G327" s="19">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="H327" s="17" t="s">
         <v>37</v>
@@ -11849,7 +11849,7 @@
         <v>36</v>
       </c>
       <c r="G328" s="19">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H328" s="17" t="s">
         <v>37</v>
@@ -11875,7 +11875,7 @@
         <v>36</v>
       </c>
       <c r="G329" s="19">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="H329" s="17" t="s">
         <v>37</v>
@@ -11901,7 +11901,7 @@
         <v>36</v>
       </c>
       <c r="G330" s="19">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H330" s="17" t="s">
         <v>37</v>
@@ -11927,7 +11927,7 @@
         <v>36</v>
       </c>
       <c r="G331" s="19">
-        <v>36</v>
+        <v>7</v>
       </c>
       <c r="H331" s="17" t="s">
         <v>37</v>
@@ -11953,7 +11953,7 @@
         <v>36</v>
       </c>
       <c r="G332" s="19">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="H332" s="17" t="s">
         <v>37</v>
@@ -11979,7 +11979,7 @@
         <v>36</v>
       </c>
       <c r="G333" s="19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H333" s="17" t="s">
         <v>37</v>
@@ -12005,7 +12005,7 @@
         <v>36</v>
       </c>
       <c r="G334" s="19">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H334" s="17" t="s">
         <v>37</v>
@@ -12031,7 +12031,7 @@
         <v>36</v>
       </c>
       <c r="G335" s="19">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H335" s="17" t="s">
         <v>37</v>
@@ -12057,7 +12057,7 @@
         <v>36</v>
       </c>
       <c r="G336" s="19">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="H336" s="17" t="s">
         <v>37</v>
@@ -12083,7 +12083,7 @@
         <v>36</v>
       </c>
       <c r="G337" s="19">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H337" s="17" t="s">
         <v>37</v>
@@ -12109,7 +12109,7 @@
         <v>36</v>
       </c>
       <c r="G338" s="19">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="H338" s="17" t="s">
         <v>37</v>
@@ -12135,7 +12135,7 @@
         <v>36</v>
       </c>
       <c r="G339" s="19">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="H339" s="17" t="s">
         <v>37</v>
@@ -12161,7 +12161,7 @@
         <v>36</v>
       </c>
       <c r="G340" s="19">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="H340" s="17" t="s">
         <v>37</v>
@@ -12187,7 +12187,7 @@
         <v>36</v>
       </c>
       <c r="G341" s="19">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="H341" s="17" t="s">
         <v>37</v>
@@ -12213,7 +12213,7 @@
         <v>36</v>
       </c>
       <c r="G342" s="19">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H342" s="17" t="s">
         <v>37</v>
@@ -12239,7 +12239,7 @@
         <v>36</v>
       </c>
       <c r="G343" s="19">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="H343" s="17" t="s">
         <v>37</v>
@@ -12265,7 +12265,7 @@
         <v>36</v>
       </c>
       <c r="G344" s="19">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H344" s="17" t="s">
         <v>37</v>
@@ -12291,7 +12291,7 @@
         <v>36</v>
       </c>
       <c r="G345" s="19">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H345" s="17" t="s">
         <v>37</v>
@@ -12317,7 +12317,7 @@
         <v>36</v>
       </c>
       <c r="G346" s="19">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H346" s="17" t="s">
         <v>37</v>
@@ -12343,7 +12343,7 @@
         <v>36</v>
       </c>
       <c r="G347" s="19">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="H347" s="17" t="s">
         <v>37</v>
@@ -12369,7 +12369,7 @@
         <v>36</v>
       </c>
       <c r="G348" s="19">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H348" s="17" t="s">
         <v>37</v>
@@ -12395,7 +12395,7 @@
         <v>36</v>
       </c>
       <c r="G349" s="19">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="H349" s="17" t="s">
         <v>37</v>
@@ -12421,7 +12421,7 @@
         <v>36</v>
       </c>
       <c r="G350" s="19">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H350" s="17" t="s">
         <v>37</v>
@@ -12447,7 +12447,7 @@
         <v>36</v>
       </c>
       <c r="G351" s="19">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H351" s="17" t="s">
         <v>37</v>
@@ -12473,7 +12473,7 @@
         <v>36</v>
       </c>
       <c r="G352" s="19">
-        <v>2</v>
+        <v>31</v>
       </c>
       <c r="H352" s="17" t="s">
         <v>37</v>
@@ -12499,7 +12499,7 @@
         <v>36</v>
       </c>
       <c r="G353" s="19">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H353" s="17" t="s">
         <v>37</v>
@@ -12525,7 +12525,7 @@
         <v>36</v>
       </c>
       <c r="G354" s="19">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H354" s="17" t="s">
         <v>37</v>
@@ -12551,7 +12551,7 @@
         <v>36</v>
       </c>
       <c r="G355" s="19">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H355" s="17" t="s">
         <v>37</v>
@@ -12577,7 +12577,7 @@
         <v>36</v>
       </c>
       <c r="G356" s="19">
-        <v>35</v>
+        <v>9</v>
       </c>
       <c r="H356" s="17" t="s">
         <v>37</v>
@@ -12603,7 +12603,7 @@
         <v>36</v>
       </c>
       <c r="G357" s="19">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="H357" s="17" t="s">
         <v>37</v>
@@ -12629,7 +12629,7 @@
         <v>36</v>
       </c>
       <c r="G358" s="19">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H358" s="17" t="s">
         <v>37</v>
@@ -12655,7 +12655,7 @@
         <v>36</v>
       </c>
       <c r="G359" s="19">
-        <v>19</v>
+        <v>1</v>
       </c>
       <c r="H359" s="17" t="s">
         <v>37</v>
@@ -12707,7 +12707,7 @@
         <v>36</v>
       </c>
       <c r="G361" s="19">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="H361" s="17" t="s">
         <v>37</v>
@@ -12733,7 +12733,7 @@
         <v>36</v>
       </c>
       <c r="G362" s="19">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H362" s="17" t="s">
         <v>37</v>
@@ -12759,7 +12759,7 @@
         <v>36</v>
       </c>
       <c r="G363" s="19">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H363" s="17" t="s">
         <v>37</v>
@@ -12785,7 +12785,7 @@
         <v>36</v>
       </c>
       <c r="G364" s="19">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H364" s="17" t="s">
         <v>37</v>
@@ -12811,7 +12811,7 @@
         <v>36</v>
       </c>
       <c r="G365" s="19">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="H365" s="17" t="s">
         <v>37</v>
@@ -12837,7 +12837,7 @@
         <v>36</v>
       </c>
       <c r="G366" s="19">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H366" s="17" t="s">
         <v>37</v>
@@ -12863,7 +12863,7 @@
         <v>36</v>
       </c>
       <c r="G367" s="19">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H367" s="17" t="s">
         <v>37</v>
@@ -12889,7 +12889,7 @@
         <v>36</v>
       </c>
       <c r="G368" s="19">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="H368" s="17" t="s">
         <v>37</v>
@@ -12915,7 +12915,7 @@
         <v>36</v>
       </c>
       <c r="G369" s="19">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H369" s="17" t="s">
         <v>37</v>
@@ -12941,7 +12941,7 @@
         <v>36</v>
       </c>
       <c r="G370" s="19">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="H370" s="17" t="s">
         <v>37</v>
@@ -12967,7 +12967,7 @@
         <v>36</v>
       </c>
       <c r="G371" s="19">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H371" s="17" t="s">
         <v>37</v>
@@ -12993,7 +12993,7 @@
         <v>36</v>
       </c>
       <c r="G372" s="19">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="H372" s="17" t="s">
         <v>37</v>
@@ -13019,7 +13019,7 @@
         <v>36</v>
       </c>
       <c r="G373" s="19">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="H373" s="17" t="s">
         <v>37</v>
@@ -13045,7 +13045,7 @@
         <v>36</v>
       </c>
       <c r="G374" s="19">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H374" s="17" t="s">
         <v>37</v>
@@ -13071,7 +13071,7 @@
         <v>36</v>
       </c>
       <c r="G375" s="19">
-        <v>3</v>
+        <v>36</v>
       </c>
       <c r="H375" s="17" t="s">
         <v>37</v>
@@ -13123,7 +13123,7 @@
         <v>36</v>
       </c>
       <c r="G377" s="19">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="H377" s="17" t="s">
         <v>37</v>
@@ -13149,7 +13149,7 @@
         <v>36</v>
       </c>
       <c r="G378" s="19">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="H378" s="17" t="s">
         <v>37</v>
@@ -13175,7 +13175,7 @@
         <v>36</v>
       </c>
       <c r="G379" s="19">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="H379" s="17" t="s">
         <v>37</v>
@@ -13201,7 +13201,7 @@
         <v>36</v>
       </c>
       <c r="G380" s="19">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="H380" s="17" t="s">
         <v>37</v>
@@ -13227,7 +13227,7 @@
         <v>36</v>
       </c>
       <c r="G381" s="19">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="H381" s="17" t="s">
         <v>37</v>
@@ -13253,7 +13253,7 @@
         <v>36</v>
       </c>
       <c r="G382" s="19">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="H382" s="17" t="s">
         <v>37</v>
@@ -13279,7 +13279,7 @@
         <v>36</v>
       </c>
       <c r="G383" s="19">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="H383" s="17" t="s">
         <v>37</v>
@@ -13305,7 +13305,7 @@
         <v>36</v>
       </c>
       <c r="G384" s="19">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="H384" s="17" t="s">
         <v>37</v>
@@ -13331,7 +13331,7 @@
         <v>36</v>
       </c>
       <c r="G385" s="19">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="H385" s="17" t="s">
         <v>37</v>
@@ -13357,7 +13357,7 @@
         <v>36</v>
       </c>
       <c r="G386" s="19">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="H386" s="17" t="s">
         <v>37</v>
@@ -13383,7 +13383,7 @@
         <v>36</v>
       </c>
       <c r="G387" s="19">
-        <v>38</v>
+        <v>5</v>
       </c>
       <c r="H387" s="17" t="s">
         <v>37</v>
@@ -13409,7 +13409,7 @@
         <v>36</v>
       </c>
       <c r="G388" s="19">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="H388" s="17" t="s">
         <v>37</v>
@@ -13435,7 +13435,7 @@
         <v>36</v>
       </c>
       <c r="G389" s="19">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="H389" s="17" t="s">
         <v>37</v>
@@ -13461,7 +13461,7 @@
         <v>36</v>
       </c>
       <c r="G390" s="19">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H390" s="17" t="s">
         <v>37</v>
@@ -13487,7 +13487,7 @@
         <v>36</v>
       </c>
       <c r="G391" s="19">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="H391" s="17" t="s">
         <v>37</v>
@@ -13513,7 +13513,7 @@
         <v>36</v>
       </c>
       <c r="G392" s="19">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="H392" s="17" t="s">
         <v>37</v>
@@ -13539,7 +13539,7 @@
         <v>36</v>
       </c>
       <c r="G393" s="19">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="H393" s="17" t="s">
         <v>37</v>
@@ -13565,7 +13565,7 @@
         <v>36</v>
       </c>
       <c r="G394" s="19">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="H394" s="17" t="s">
         <v>37</v>
@@ -13591,7 +13591,7 @@
         <v>36</v>
       </c>
       <c r="G395" s="19">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H395" s="17" t="s">
         <v>37</v>
@@ -13617,7 +13617,7 @@
         <v>36</v>
       </c>
       <c r="G396" s="19">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H396" s="17" t="s">
         <v>37</v>
@@ -13643,7 +13643,7 @@
         <v>36</v>
       </c>
       <c r="G397" s="19">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="H397" s="17" t="s">
         <v>37</v>
@@ -13695,7 +13695,7 @@
         <v>36</v>
       </c>
       <c r="G399" s="19">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="H399" s="17" t="s">
         <v>37</v>
@@ -13721,7 +13721,7 @@
         <v>36</v>
       </c>
       <c r="G400" s="19">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="H400" s="17" t="s">
         <v>37</v>
@@ -13747,7 +13747,7 @@
         <v>36</v>
       </c>
       <c r="G401" s="19">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="H401" s="17" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
📊 Consolidated Test Report – Build #3 fcd2ef6c9ec82132ed562252f89453922bddacd1
</commit_message>
<xml_diff>
--- a/backend-reports/functional-test-report.xlsx
+++ b/backend-reports/functional-test-report.xlsx
@@ -83,7 +83,7 @@
     <t>Date &amp; Time</t>
   </si>
   <si>
-    <t>7/19/2026, 5:56:26 PM</t>
+    <t>7/19/2026, 6:21:22 PM</t>
   </si>
   <si>
     <t>Duration</t>
@@ -3373,7 +3373,7 @@
         <v>36</v>
       </c>
       <c r="G2" s="19">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H2" s="17" t="s">
         <v>37</v>
@@ -3399,7 +3399,7 @@
         <v>36</v>
       </c>
       <c r="G3" s="19">
-        <v>23</v>
+        <v>36</v>
       </c>
       <c r="H3" s="17" t="s">
         <v>37</v>
@@ -3425,7 +3425,7 @@
         <v>36</v>
       </c>
       <c r="G4" s="19">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>37</v>
@@ -3451,7 +3451,7 @@
         <v>36</v>
       </c>
       <c r="G5" s="19">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>37</v>
@@ -3477,7 +3477,7 @@
         <v>36</v>
       </c>
       <c r="G6" s="19">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>37</v>
@@ -3503,7 +3503,7 @@
         <v>36</v>
       </c>
       <c r="G7" s="19">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>37</v>
@@ -3529,7 +3529,7 @@
         <v>36</v>
       </c>
       <c r="G8" s="19">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>37</v>
@@ -3555,7 +3555,7 @@
         <v>36</v>
       </c>
       <c r="G9" s="19">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>37</v>
@@ -3581,7 +3581,7 @@
         <v>36</v>
       </c>
       <c r="G10" s="19">
-        <v>34</v>
+        <v>14</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>37</v>
@@ -3607,7 +3607,7 @@
         <v>36</v>
       </c>
       <c r="G11" s="19">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>37</v>
@@ -3633,7 +3633,7 @@
         <v>36</v>
       </c>
       <c r="G12" s="19">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>37</v>
@@ -3659,7 +3659,7 @@
         <v>36</v>
       </c>
       <c r="G13" s="19">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>37</v>
@@ -3685,7 +3685,7 @@
         <v>36</v>
       </c>
       <c r="G14" s="19">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>37</v>
@@ -3711,7 +3711,7 @@
         <v>36</v>
       </c>
       <c r="G15" s="19">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H15" s="17" t="s">
         <v>37</v>
@@ -3737,7 +3737,7 @@
         <v>36</v>
       </c>
       <c r="G16" s="19">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>37</v>
@@ -3763,7 +3763,7 @@
         <v>36</v>
       </c>
       <c r="G17" s="19">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="H17" s="17" t="s">
         <v>37</v>
@@ -3789,7 +3789,7 @@
         <v>36</v>
       </c>
       <c r="G18" s="19">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="H18" s="17" t="s">
         <v>37</v>
@@ -3815,7 +3815,7 @@
         <v>36</v>
       </c>
       <c r="G19" s="19">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="H19" s="17" t="s">
         <v>37</v>
@@ -3841,7 +3841,7 @@
         <v>36</v>
       </c>
       <c r="G20" s="19">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="H20" s="17" t="s">
         <v>37</v>
@@ -3867,7 +3867,7 @@
         <v>36</v>
       </c>
       <c r="G21" s="19">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="H21" s="17" t="s">
         <v>37</v>
@@ -3893,7 +3893,7 @@
         <v>36</v>
       </c>
       <c r="G22" s="19">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="H22" s="17" t="s">
         <v>37</v>
@@ -3919,7 +3919,7 @@
         <v>36</v>
       </c>
       <c r="G23" s="19">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="H23" s="17" t="s">
         <v>37</v>
@@ -3945,7 +3945,7 @@
         <v>36</v>
       </c>
       <c r="G24" s="19">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H24" s="17" t="s">
         <v>37</v>
@@ -3971,7 +3971,7 @@
         <v>36</v>
       </c>
       <c r="G25" s="19">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="H25" s="17" t="s">
         <v>37</v>
@@ -4023,7 +4023,7 @@
         <v>36</v>
       </c>
       <c r="G27" s="19">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H27" s="17" t="s">
         <v>37</v>
@@ -4049,7 +4049,7 @@
         <v>36</v>
       </c>
       <c r="G28" s="19">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="H28" s="17" t="s">
         <v>37</v>
@@ -4075,7 +4075,7 @@
         <v>36</v>
       </c>
       <c r="G29" s="19">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H29" s="17" t="s">
         <v>37</v>
@@ -4101,7 +4101,7 @@
         <v>36</v>
       </c>
       <c r="G30" s="19">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="H30" s="17" t="s">
         <v>37</v>
@@ -4127,7 +4127,7 @@
         <v>36</v>
       </c>
       <c r="G31" s="19">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H31" s="17" t="s">
         <v>37</v>
@@ -4153,7 +4153,7 @@
         <v>36</v>
       </c>
       <c r="G32" s="19">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H32" s="17" t="s">
         <v>37</v>
@@ -4179,7 +4179,7 @@
         <v>36</v>
       </c>
       <c r="G33" s="19">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="H33" s="17" t="s">
         <v>37</v>
@@ -4205,7 +4205,7 @@
         <v>36</v>
       </c>
       <c r="G34" s="19">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="H34" s="17" t="s">
         <v>37</v>
@@ -4231,7 +4231,7 @@
         <v>36</v>
       </c>
       <c r="G35" s="19">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="H35" s="17" t="s">
         <v>37</v>
@@ -4257,7 +4257,7 @@
         <v>36</v>
       </c>
       <c r="G36" s="19">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="H36" s="17" t="s">
         <v>37</v>
@@ -4283,7 +4283,7 @@
         <v>36</v>
       </c>
       <c r="G37" s="19">
-        <v>39</v>
+        <v>10</v>
       </c>
       <c r="H37" s="17" t="s">
         <v>37</v>
@@ -4309,7 +4309,7 @@
         <v>36</v>
       </c>
       <c r="G38" s="19">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="H38" s="17" t="s">
         <v>37</v>
@@ -4335,7 +4335,7 @@
         <v>36</v>
       </c>
       <c r="G39" s="19">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="H39" s="17" t="s">
         <v>37</v>
@@ -4361,7 +4361,7 @@
         <v>36</v>
       </c>
       <c r="G40" s="19">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="H40" s="17" t="s">
         <v>37</v>
@@ -4387,7 +4387,7 @@
         <v>36</v>
       </c>
       <c r="G41" s="19">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="H41" s="17" t="s">
         <v>37</v>
@@ -4413,7 +4413,7 @@
         <v>36</v>
       </c>
       <c r="G42" s="19">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>37</v>
@@ -4439,7 +4439,7 @@
         <v>36</v>
       </c>
       <c r="G43" s="19">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H43" s="17" t="s">
         <v>37</v>
@@ -4465,7 +4465,7 @@
         <v>36</v>
       </c>
       <c r="G44" s="19">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H44" s="17" t="s">
         <v>37</v>
@@ -4491,7 +4491,7 @@
         <v>36</v>
       </c>
       <c r="G45" s="19">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H45" s="17" t="s">
         <v>37</v>
@@ -4517,7 +4517,7 @@
         <v>36</v>
       </c>
       <c r="G46" s="19">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H46" s="17" t="s">
         <v>37</v>
@@ -4543,7 +4543,7 @@
         <v>36</v>
       </c>
       <c r="G47" s="19">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="H47" s="17" t="s">
         <v>37</v>
@@ -4569,7 +4569,7 @@
         <v>36</v>
       </c>
       <c r="G48" s="19">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H48" s="17" t="s">
         <v>37</v>
@@ -4595,7 +4595,7 @@
         <v>36</v>
       </c>
       <c r="G49" s="19">
-        <v>2</v>
+        <v>28</v>
       </c>
       <c r="H49" s="17" t="s">
         <v>37</v>
@@ -4621,7 +4621,7 @@
         <v>36</v>
       </c>
       <c r="G50" s="19">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H50" s="17" t="s">
         <v>37</v>
@@ -4647,7 +4647,7 @@
         <v>36</v>
       </c>
       <c r="G51" s="19">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H51" s="17" t="s">
         <v>37</v>
@@ -4673,7 +4673,7 @@
         <v>36</v>
       </c>
       <c r="G52" s="19">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H52" s="17" t="s">
         <v>37</v>
@@ -4699,7 +4699,7 @@
         <v>36</v>
       </c>
       <c r="G53" s="19">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="H53" s="17" t="s">
         <v>37</v>
@@ -4751,7 +4751,7 @@
         <v>36</v>
       </c>
       <c r="G55" s="19">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H55" s="17" t="s">
         <v>37</v>
@@ -4777,7 +4777,7 @@
         <v>36</v>
       </c>
       <c r="G56" s="19">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="H56" s="17" t="s">
         <v>37</v>
@@ -4803,7 +4803,7 @@
         <v>36</v>
       </c>
       <c r="G57" s="19">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="H57" s="17" t="s">
         <v>37</v>
@@ -4829,7 +4829,7 @@
         <v>36</v>
       </c>
       <c r="G58" s="19">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="H58" s="17" t="s">
         <v>37</v>
@@ -4855,7 +4855,7 @@
         <v>36</v>
       </c>
       <c r="G59" s="19">
-        <v>5</v>
+        <v>24</v>
       </c>
       <c r="H59" s="17" t="s">
         <v>37</v>
@@ -4881,7 +4881,7 @@
         <v>36</v>
       </c>
       <c r="G60" s="19">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="H60" s="17" t="s">
         <v>37</v>
@@ -4933,7 +4933,7 @@
         <v>36</v>
       </c>
       <c r="G62" s="19">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H62" s="17" t="s">
         <v>37</v>
@@ -4959,7 +4959,7 @@
         <v>36</v>
       </c>
       <c r="G63" s="19">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="H63" s="17" t="s">
         <v>37</v>
@@ -4985,7 +4985,7 @@
         <v>36</v>
       </c>
       <c r="G64" s="19">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="H64" s="17" t="s">
         <v>37</v>
@@ -5011,7 +5011,7 @@
         <v>36</v>
       </c>
       <c r="G65" s="19">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H65" s="17" t="s">
         <v>37</v>
@@ -5037,7 +5037,7 @@
         <v>36</v>
       </c>
       <c r="G66" s="19">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H66" s="17" t="s">
         <v>37</v>
@@ -5063,7 +5063,7 @@
         <v>36</v>
       </c>
       <c r="G67" s="19">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H67" s="17" t="s">
         <v>37</v>
@@ -5089,7 +5089,7 @@
         <v>36</v>
       </c>
       <c r="G68" s="19">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="H68" s="17" t="s">
         <v>37</v>
@@ -5115,7 +5115,7 @@
         <v>36</v>
       </c>
       <c r="G69" s="19">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="H69" s="17" t="s">
         <v>37</v>
@@ -5141,7 +5141,7 @@
         <v>36</v>
       </c>
       <c r="G70" s="19">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H70" s="17" t="s">
         <v>37</v>
@@ -5193,7 +5193,7 @@
         <v>36</v>
       </c>
       <c r="G72" s="19">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="H72" s="17" t="s">
         <v>37</v>
@@ -5219,7 +5219,7 @@
         <v>36</v>
       </c>
       <c r="G73" s="19">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="H73" s="17" t="s">
         <v>37</v>
@@ -5245,7 +5245,7 @@
         <v>36</v>
       </c>
       <c r="G74" s="19">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="H74" s="17" t="s">
         <v>37</v>
@@ -5271,7 +5271,7 @@
         <v>36</v>
       </c>
       <c r="G75" s="19">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="H75" s="17" t="s">
         <v>37</v>
@@ -5297,7 +5297,7 @@
         <v>36</v>
       </c>
       <c r="G76" s="19">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="H76" s="17" t="s">
         <v>37</v>
@@ -5323,7 +5323,7 @@
         <v>36</v>
       </c>
       <c r="G77" s="19">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="H77" s="17" t="s">
         <v>37</v>
@@ -5349,7 +5349,7 @@
         <v>36</v>
       </c>
       <c r="G78" s="19">
-        <v>21</v>
+        <v>4</v>
       </c>
       <c r="H78" s="17" t="s">
         <v>37</v>
@@ -5375,7 +5375,7 @@
         <v>36</v>
       </c>
       <c r="G79" s="19">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="H79" s="17" t="s">
         <v>37</v>
@@ -5401,7 +5401,7 @@
         <v>36</v>
       </c>
       <c r="G80" s="19">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="H80" s="17" t="s">
         <v>37</v>
@@ -5427,7 +5427,7 @@
         <v>36</v>
       </c>
       <c r="G81" s="19">
-        <v>7</v>
+        <v>25</v>
       </c>
       <c r="H81" s="17" t="s">
         <v>37</v>
@@ -5453,7 +5453,7 @@
         <v>36</v>
       </c>
       <c r="G82" s="19">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="H82" s="17" t="s">
         <v>37</v>
@@ -5479,7 +5479,7 @@
         <v>36</v>
       </c>
       <c r="G83" s="19">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="H83" s="17" t="s">
         <v>37</v>
@@ -5505,7 +5505,7 @@
         <v>36</v>
       </c>
       <c r="G84" s="19">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="H84" s="17" t="s">
         <v>37</v>
@@ -5531,7 +5531,7 @@
         <v>36</v>
       </c>
       <c r="G85" s="19">
-        <v>35</v>
+        <v>24</v>
       </c>
       <c r="H85" s="17" t="s">
         <v>37</v>
@@ -5557,7 +5557,7 @@
         <v>36</v>
       </c>
       <c r="G86" s="19">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="H86" s="17" t="s">
         <v>37</v>
@@ -5583,7 +5583,7 @@
         <v>36</v>
       </c>
       <c r="G87" s="19">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="H87" s="17" t="s">
         <v>37</v>
@@ -5609,7 +5609,7 @@
         <v>36</v>
       </c>
       <c r="G88" s="19">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="H88" s="17" t="s">
         <v>37</v>
@@ -5661,7 +5661,7 @@
         <v>36</v>
       </c>
       <c r="G90" s="19">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="H90" s="17" t="s">
         <v>37</v>
@@ -5687,7 +5687,7 @@
         <v>36</v>
       </c>
       <c r="G91" s="19">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H91" s="17" t="s">
         <v>37</v>
@@ -5713,7 +5713,7 @@
         <v>36</v>
       </c>
       <c r="G92" s="19">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H92" s="17" t="s">
         <v>37</v>
@@ -5739,7 +5739,7 @@
         <v>36</v>
       </c>
       <c r="G93" s="19">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="H93" s="17" t="s">
         <v>37</v>
@@ -5765,7 +5765,7 @@
         <v>36</v>
       </c>
       <c r="G94" s="19">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="H94" s="17" t="s">
         <v>37</v>
@@ -5791,7 +5791,7 @@
         <v>36</v>
       </c>
       <c r="G95" s="19">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="H95" s="17" t="s">
         <v>37</v>
@@ -5817,7 +5817,7 @@
         <v>36</v>
       </c>
       <c r="G96" s="19">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="H96" s="17" t="s">
         <v>37</v>
@@ -5843,7 +5843,7 @@
         <v>36</v>
       </c>
       <c r="G97" s="19">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="H97" s="17" t="s">
         <v>37</v>
@@ -5869,7 +5869,7 @@
         <v>36</v>
       </c>
       <c r="G98" s="19">
-        <v>39</v>
+        <v>17</v>
       </c>
       <c r="H98" s="17" t="s">
         <v>37</v>
@@ -5895,7 +5895,7 @@
         <v>36</v>
       </c>
       <c r="G99" s="19">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="H99" s="17" t="s">
         <v>37</v>
@@ -5921,7 +5921,7 @@
         <v>36</v>
       </c>
       <c r="G100" s="19">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="H100" s="17" t="s">
         <v>37</v>
@@ -5947,7 +5947,7 @@
         <v>36</v>
       </c>
       <c r="G101" s="19">
-        <v>31</v>
+        <v>11</v>
       </c>
       <c r="H101" s="17" t="s">
         <v>37</v>
@@ -5973,7 +5973,7 @@
         <v>36</v>
       </c>
       <c r="G102" s="19">
-        <v>12</v>
+        <v>24</v>
       </c>
       <c r="H102" s="17" t="s">
         <v>37</v>
@@ -5999,7 +5999,7 @@
         <v>36</v>
       </c>
       <c r="G103" s="19">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="H103" s="17" t="s">
         <v>37</v>
@@ -6025,7 +6025,7 @@
         <v>36</v>
       </c>
       <c r="G104" s="19">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="H104" s="17" t="s">
         <v>37</v>
@@ -6051,7 +6051,7 @@
         <v>36</v>
       </c>
       <c r="G105" s="19">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H105" s="17" t="s">
         <v>37</v>
@@ -6077,7 +6077,7 @@
         <v>36</v>
       </c>
       <c r="G106" s="19">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="H106" s="17" t="s">
         <v>37</v>
@@ -6103,7 +6103,7 @@
         <v>36</v>
       </c>
       <c r="G107" s="19">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="H107" s="17" t="s">
         <v>37</v>
@@ -6129,7 +6129,7 @@
         <v>36</v>
       </c>
       <c r="G108" s="19">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c r="H108" s="17" t="s">
         <v>37</v>
@@ -6155,7 +6155,7 @@
         <v>36</v>
       </c>
       <c r="G109" s="19">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="H109" s="17" t="s">
         <v>37</v>
@@ -6181,7 +6181,7 @@
         <v>36</v>
       </c>
       <c r="G110" s="19">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H110" s="17" t="s">
         <v>37</v>
@@ -6207,7 +6207,7 @@
         <v>36</v>
       </c>
       <c r="G111" s="19">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H111" s="17" t="s">
         <v>37</v>
@@ -6233,7 +6233,7 @@
         <v>36</v>
       </c>
       <c r="G112" s="19">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="H112" s="17" t="s">
         <v>37</v>
@@ -6259,7 +6259,7 @@
         <v>36</v>
       </c>
       <c r="G113" s="19">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="H113" s="17" t="s">
         <v>37</v>
@@ -6285,7 +6285,7 @@
         <v>36</v>
       </c>
       <c r="G114" s="19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H114" s="17" t="s">
         <v>37</v>
@@ -6311,7 +6311,7 @@
         <v>36</v>
       </c>
       <c r="G115" s="19">
-        <v>35</v>
+        <v>23</v>
       </c>
       <c r="H115" s="17" t="s">
         <v>37</v>
@@ -6337,7 +6337,7 @@
         <v>36</v>
       </c>
       <c r="G116" s="19">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H116" s="17" t="s">
         <v>37</v>
@@ -6363,7 +6363,7 @@
         <v>36</v>
       </c>
       <c r="G117" s="19">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="H117" s="17" t="s">
         <v>37</v>
@@ -6389,7 +6389,7 @@
         <v>36</v>
       </c>
       <c r="G118" s="19">
-        <v>11</v>
+        <v>5</v>
       </c>
       <c r="H118" s="17" t="s">
         <v>37</v>
@@ -6415,7 +6415,7 @@
         <v>36</v>
       </c>
       <c r="G119" s="19">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="H119" s="17" t="s">
         <v>37</v>
@@ -6441,7 +6441,7 @@
         <v>36</v>
       </c>
       <c r="G120" s="19">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="H120" s="17" t="s">
         <v>37</v>
@@ -6467,7 +6467,7 @@
         <v>36</v>
       </c>
       <c r="G121" s="19">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H121" s="17" t="s">
         <v>37</v>
@@ -6493,7 +6493,7 @@
         <v>36</v>
       </c>
       <c r="G122" s="19">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H122" s="17" t="s">
         <v>37</v>
@@ -6519,7 +6519,7 @@
         <v>36</v>
       </c>
       <c r="G123" s="19">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="H123" s="17" t="s">
         <v>37</v>
@@ -6545,7 +6545,7 @@
         <v>36</v>
       </c>
       <c r="G124" s="19">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H124" s="17" t="s">
         <v>37</v>
@@ -6571,7 +6571,7 @@
         <v>36</v>
       </c>
       <c r="G125" s="19">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H125" s="17" t="s">
         <v>37</v>
@@ -6597,7 +6597,7 @@
         <v>36</v>
       </c>
       <c r="G126" s="19">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="H126" s="17" t="s">
         <v>37</v>
@@ -6623,7 +6623,7 @@
         <v>36</v>
       </c>
       <c r="G127" s="19">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H127" s="17" t="s">
         <v>37</v>
@@ -6649,7 +6649,7 @@
         <v>36</v>
       </c>
       <c r="G128" s="19">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H128" s="17" t="s">
         <v>37</v>
@@ -6675,7 +6675,7 @@
         <v>36</v>
       </c>
       <c r="G129" s="19">
-        <v>3</v>
+        <v>33</v>
       </c>
       <c r="H129" s="17" t="s">
         <v>37</v>
@@ -6701,7 +6701,7 @@
         <v>36</v>
       </c>
       <c r="G130" s="19">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H130" s="17" t="s">
         <v>37</v>
@@ -6727,7 +6727,7 @@
         <v>36</v>
       </c>
       <c r="G131" s="19">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="H131" s="17" t="s">
         <v>37</v>
@@ -6753,7 +6753,7 @@
         <v>36</v>
       </c>
       <c r="G132" s="19">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="H132" s="17" t="s">
         <v>37</v>
@@ -6779,7 +6779,7 @@
         <v>36</v>
       </c>
       <c r="G133" s="19">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="H133" s="17" t="s">
         <v>37</v>
@@ -6805,7 +6805,7 @@
         <v>36</v>
       </c>
       <c r="G134" s="19">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="H134" s="17" t="s">
         <v>37</v>
@@ -6831,7 +6831,7 @@
         <v>36</v>
       </c>
       <c r="G135" s="19">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H135" s="17" t="s">
         <v>37</v>
@@ -6857,7 +6857,7 @@
         <v>36</v>
       </c>
       <c r="G136" s="19">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="H136" s="17" t="s">
         <v>37</v>
@@ -6883,7 +6883,7 @@
         <v>36</v>
       </c>
       <c r="G137" s="19">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="H137" s="17" t="s">
         <v>37</v>
@@ -6909,7 +6909,7 @@
         <v>36</v>
       </c>
       <c r="G138" s="19">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="H138" s="17" t="s">
         <v>37</v>
@@ -6935,7 +6935,7 @@
         <v>36</v>
       </c>
       <c r="G139" s="19">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H139" s="17" t="s">
         <v>37</v>
@@ -6961,7 +6961,7 @@
         <v>36</v>
       </c>
       <c r="G140" s="19">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="H140" s="17" t="s">
         <v>37</v>
@@ -6987,7 +6987,7 @@
         <v>36</v>
       </c>
       <c r="G141" s="19">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H141" s="17" t="s">
         <v>37</v>
@@ -7013,7 +7013,7 @@
         <v>36</v>
       </c>
       <c r="G142" s="19">
-        <v>26</v>
+        <v>11</v>
       </c>
       <c r="H142" s="17" t="s">
         <v>37</v>
@@ -7039,7 +7039,7 @@
         <v>36</v>
       </c>
       <c r="G143" s="19">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H143" s="17" t="s">
         <v>37</v>
@@ -7065,7 +7065,7 @@
         <v>36</v>
       </c>
       <c r="G144" s="19">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H144" s="17" t="s">
         <v>37</v>
@@ -7091,7 +7091,7 @@
         <v>36</v>
       </c>
       <c r="G145" s="19">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="H145" s="17" t="s">
         <v>37</v>
@@ -7117,7 +7117,7 @@
         <v>36</v>
       </c>
       <c r="G146" s="19">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="H146" s="17" t="s">
         <v>37</v>
@@ -7143,7 +7143,7 @@
         <v>36</v>
       </c>
       <c r="G147" s="19">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="H147" s="17" t="s">
         <v>37</v>
@@ -7169,7 +7169,7 @@
         <v>36</v>
       </c>
       <c r="G148" s="19">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H148" s="17" t="s">
         <v>37</v>
@@ -7195,7 +7195,7 @@
         <v>36</v>
       </c>
       <c r="G149" s="19">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="H149" s="17" t="s">
         <v>37</v>
@@ -7221,7 +7221,7 @@
         <v>36</v>
       </c>
       <c r="G150" s="19">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H150" s="17" t="s">
         <v>37</v>
@@ -7247,7 +7247,7 @@
         <v>36</v>
       </c>
       <c r="G151" s="19">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H151" s="17" t="s">
         <v>37</v>
@@ -7273,7 +7273,7 @@
         <v>36</v>
       </c>
       <c r="G152" s="19">
-        <v>38</v>
+        <v>25</v>
       </c>
       <c r="H152" s="17" t="s">
         <v>37</v>
@@ -7299,7 +7299,7 @@
         <v>36</v>
       </c>
       <c r="G153" s="19">
-        <v>26</v>
+        <v>3</v>
       </c>
       <c r="H153" s="17" t="s">
         <v>37</v>
@@ -7325,7 +7325,7 @@
         <v>36</v>
       </c>
       <c r="G154" s="19">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H154" s="17" t="s">
         <v>37</v>
@@ -7351,7 +7351,7 @@
         <v>36</v>
       </c>
       <c r="G155" s="19">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="H155" s="17" t="s">
         <v>37</v>
@@ -7377,7 +7377,7 @@
         <v>36</v>
       </c>
       <c r="G156" s="19">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="H156" s="17" t="s">
         <v>37</v>
@@ -7403,7 +7403,7 @@
         <v>36</v>
       </c>
       <c r="G157" s="19">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="H157" s="17" t="s">
         <v>37</v>
@@ -7429,7 +7429,7 @@
         <v>36</v>
       </c>
       <c r="G158" s="19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H158" s="17" t="s">
         <v>37</v>
@@ -7455,7 +7455,7 @@
         <v>36</v>
       </c>
       <c r="G159" s="19">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="H159" s="17" t="s">
         <v>37</v>
@@ -7481,7 +7481,7 @@
         <v>36</v>
       </c>
       <c r="G160" s="19">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="H160" s="17" t="s">
         <v>37</v>
@@ -7507,7 +7507,7 @@
         <v>36</v>
       </c>
       <c r="G161" s="19">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H161" s="17" t="s">
         <v>37</v>
@@ -7533,7 +7533,7 @@
         <v>36</v>
       </c>
       <c r="G162" s="19">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="H162" s="17" t="s">
         <v>37</v>
@@ -7559,7 +7559,7 @@
         <v>36</v>
       </c>
       <c r="G163" s="19">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="H163" s="17" t="s">
         <v>37</v>
@@ -7585,7 +7585,7 @@
         <v>36</v>
       </c>
       <c r="G164" s="19">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="H164" s="17" t="s">
         <v>37</v>
@@ -7637,7 +7637,7 @@
         <v>36</v>
       </c>
       <c r="G166" s="19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H166" s="17" t="s">
         <v>37</v>
@@ -7663,7 +7663,7 @@
         <v>36</v>
       </c>
       <c r="G167" s="19">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="H167" s="17" t="s">
         <v>37</v>
@@ -7689,7 +7689,7 @@
         <v>36</v>
       </c>
       <c r="G168" s="19">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H168" s="17" t="s">
         <v>37</v>
@@ -7715,7 +7715,7 @@
         <v>36</v>
       </c>
       <c r="G169" s="19">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="H169" s="17" t="s">
         <v>37</v>
@@ -7741,7 +7741,7 @@
         <v>36</v>
       </c>
       <c r="G170" s="19">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="H170" s="17" t="s">
         <v>37</v>
@@ -7767,7 +7767,7 @@
         <v>36</v>
       </c>
       <c r="G171" s="19">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="H171" s="17" t="s">
         <v>37</v>
@@ -7793,7 +7793,7 @@
         <v>36</v>
       </c>
       <c r="G172" s="19">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H172" s="17" t="s">
         <v>37</v>
@@ -7819,7 +7819,7 @@
         <v>36</v>
       </c>
       <c r="G173" s="19">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="H173" s="17" t="s">
         <v>37</v>
@@ -7845,7 +7845,7 @@
         <v>36</v>
       </c>
       <c r="G174" s="19">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="H174" s="17" t="s">
         <v>37</v>
@@ -7871,7 +7871,7 @@
         <v>36</v>
       </c>
       <c r="G175" s="19">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H175" s="17" t="s">
         <v>37</v>
@@ -7923,7 +7923,7 @@
         <v>36</v>
       </c>
       <c r="G177" s="19">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H177" s="17" t="s">
         <v>37</v>
@@ -7949,7 +7949,7 @@
         <v>36</v>
       </c>
       <c r="G178" s="19">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="H178" s="17" t="s">
         <v>37</v>
@@ -8001,7 +8001,7 @@
         <v>36</v>
       </c>
       <c r="G180" s="19">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="H180" s="17" t="s">
         <v>37</v>
@@ -8027,7 +8027,7 @@
         <v>36</v>
       </c>
       <c r="G181" s="19">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="H181" s="17" t="s">
         <v>37</v>
@@ -8053,7 +8053,7 @@
         <v>36</v>
       </c>
       <c r="G182" s="19">
-        <v>27</v>
+        <v>39</v>
       </c>
       <c r="H182" s="17" t="s">
         <v>37</v>
@@ -8079,7 +8079,7 @@
         <v>36</v>
       </c>
       <c r="G183" s="19">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="H183" s="17" t="s">
         <v>37</v>
@@ -8105,7 +8105,7 @@
         <v>36</v>
       </c>
       <c r="G184" s="19">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="H184" s="17" t="s">
         <v>37</v>
@@ -8131,7 +8131,7 @@
         <v>36</v>
       </c>
       <c r="G185" s="19">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="H185" s="17" t="s">
         <v>37</v>
@@ -8157,7 +8157,7 @@
         <v>36</v>
       </c>
       <c r="G186" s="19">
-        <v>2</v>
+        <v>14</v>
       </c>
       <c r="H186" s="17" t="s">
         <v>37</v>
@@ -8183,7 +8183,7 @@
         <v>36</v>
       </c>
       <c r="G187" s="19">
-        <v>31</v>
+        <v>13</v>
       </c>
       <c r="H187" s="17" t="s">
         <v>37</v>
@@ -8209,7 +8209,7 @@
         <v>36</v>
       </c>
       <c r="G188" s="19">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="H188" s="17" t="s">
         <v>37</v>
@@ -8235,7 +8235,7 @@
         <v>36</v>
       </c>
       <c r="G189" s="19">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H189" s="17" t="s">
         <v>37</v>
@@ -8261,7 +8261,7 @@
         <v>36</v>
       </c>
       <c r="G190" s="19">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="H190" s="17" t="s">
         <v>37</v>
@@ -8287,7 +8287,7 @@
         <v>36</v>
       </c>
       <c r="G191" s="19">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H191" s="17" t="s">
         <v>37</v>
@@ -8313,7 +8313,7 @@
         <v>36</v>
       </c>
       <c r="G192" s="19">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H192" s="17" t="s">
         <v>37</v>
@@ -8339,7 +8339,7 @@
         <v>36</v>
       </c>
       <c r="G193" s="19">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H193" s="17" t="s">
         <v>37</v>
@@ -8365,7 +8365,7 @@
         <v>36</v>
       </c>
       <c r="G194" s="19">
-        <v>19</v>
+        <v>35</v>
       </c>
       <c r="H194" s="17" t="s">
         <v>37</v>
@@ -8391,7 +8391,7 @@
         <v>36</v>
       </c>
       <c r="G195" s="19">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="H195" s="17" t="s">
         <v>37</v>
@@ -8417,7 +8417,7 @@
         <v>36</v>
       </c>
       <c r="G196" s="19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H196" s="17" t="s">
         <v>37</v>
@@ -8443,7 +8443,7 @@
         <v>36</v>
       </c>
       <c r="G197" s="19">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H197" s="17" t="s">
         <v>37</v>
@@ -8469,7 +8469,7 @@
         <v>36</v>
       </c>
       <c r="G198" s="19">
-        <v>39</v>
+        <v>5</v>
       </c>
       <c r="H198" s="17" t="s">
         <v>37</v>
@@ -8495,7 +8495,7 @@
         <v>36</v>
       </c>
       <c r="G199" s="19">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="H199" s="17" t="s">
         <v>37</v>
@@ -8521,7 +8521,7 @@
         <v>36</v>
       </c>
       <c r="G200" s="19">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="H200" s="17" t="s">
         <v>37</v>
@@ -8547,7 +8547,7 @@
         <v>36</v>
       </c>
       <c r="G201" s="19">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="H201" s="17" t="s">
         <v>37</v>
@@ -8573,7 +8573,7 @@
         <v>36</v>
       </c>
       <c r="G202" s="19">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H202" s="17" t="s">
         <v>37</v>
@@ -8599,7 +8599,7 @@
         <v>36</v>
       </c>
       <c r="G203" s="19">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H203" s="17" t="s">
         <v>37</v>
@@ -8651,7 +8651,7 @@
         <v>36</v>
       </c>
       <c r="G205" s="19">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H205" s="17" t="s">
         <v>37</v>
@@ -8677,7 +8677,7 @@
         <v>36</v>
       </c>
       <c r="G206" s="19">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="H206" s="17" t="s">
         <v>37</v>
@@ -8703,7 +8703,7 @@
         <v>36</v>
       </c>
       <c r="G207" s="19">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H207" s="17" t="s">
         <v>37</v>
@@ -8729,7 +8729,7 @@
         <v>36</v>
       </c>
       <c r="G208" s="19">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="H208" s="17" t="s">
         <v>37</v>
@@ -8755,7 +8755,7 @@
         <v>36</v>
       </c>
       <c r="G209" s="19">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="H209" s="17" t="s">
         <v>37</v>
@@ -8781,7 +8781,7 @@
         <v>36</v>
       </c>
       <c r="G210" s="19">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="H210" s="17" t="s">
         <v>37</v>
@@ -8807,7 +8807,7 @@
         <v>36</v>
       </c>
       <c r="G211" s="19">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H211" s="17" t="s">
         <v>37</v>
@@ -8833,7 +8833,7 @@
         <v>36</v>
       </c>
       <c r="G212" s="19">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="H212" s="17" t="s">
         <v>37</v>
@@ -8859,7 +8859,7 @@
         <v>36</v>
       </c>
       <c r="G213" s="19">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H213" s="17" t="s">
         <v>37</v>
@@ -8885,7 +8885,7 @@
         <v>36</v>
       </c>
       <c r="G214" s="19">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H214" s="17" t="s">
         <v>37</v>
@@ -8911,7 +8911,7 @@
         <v>36</v>
       </c>
       <c r="G215" s="19">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H215" s="17" t="s">
         <v>37</v>
@@ -8937,7 +8937,7 @@
         <v>36</v>
       </c>
       <c r="G216" s="19">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H216" s="17" t="s">
         <v>37</v>
@@ -8963,7 +8963,7 @@
         <v>36</v>
       </c>
       <c r="G217" s="19">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="H217" s="17" t="s">
         <v>37</v>
@@ -8989,7 +8989,7 @@
         <v>36</v>
       </c>
       <c r="G218" s="19">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H218" s="17" t="s">
         <v>37</v>
@@ -9015,7 +9015,7 @@
         <v>36</v>
       </c>
       <c r="G219" s="19">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H219" s="17" t="s">
         <v>37</v>
@@ -9067,7 +9067,7 @@
         <v>36</v>
       </c>
       <c r="G221" s="19">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="H221" s="17" t="s">
         <v>37</v>
@@ -9093,7 +9093,7 @@
         <v>36</v>
       </c>
       <c r="G222" s="19">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="H222" s="17" t="s">
         <v>37</v>
@@ -9119,7 +9119,7 @@
         <v>36</v>
       </c>
       <c r="G223" s="19">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H223" s="17" t="s">
         <v>37</v>
@@ -9145,7 +9145,7 @@
         <v>36</v>
       </c>
       <c r="G224" s="19">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="H224" s="17" t="s">
         <v>37</v>
@@ -9171,7 +9171,7 @@
         <v>36</v>
       </c>
       <c r="G225" s="19">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="H225" s="17" t="s">
         <v>37</v>
@@ -9197,7 +9197,7 @@
         <v>36</v>
       </c>
       <c r="G226" s="19">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H226" s="17" t="s">
         <v>37</v>
@@ -9223,7 +9223,7 @@
         <v>36</v>
       </c>
       <c r="G227" s="19">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="H227" s="17" t="s">
         <v>37</v>
@@ -9249,7 +9249,7 @@
         <v>36</v>
       </c>
       <c r="G228" s="19">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="H228" s="17" t="s">
         <v>37</v>
@@ -9275,7 +9275,7 @@
         <v>36</v>
       </c>
       <c r="G229" s="19">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H229" s="17" t="s">
         <v>37</v>
@@ -9301,7 +9301,7 @@
         <v>36</v>
       </c>
       <c r="G230" s="19">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="H230" s="17" t="s">
         <v>37</v>
@@ -9327,7 +9327,7 @@
         <v>36</v>
       </c>
       <c r="G231" s="19">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H231" s="17" t="s">
         <v>37</v>
@@ -9353,7 +9353,7 @@
         <v>36</v>
       </c>
       <c r="G232" s="19">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="H232" s="17" t="s">
         <v>37</v>
@@ -9379,7 +9379,7 @@
         <v>36</v>
       </c>
       <c r="G233" s="19">
-        <v>14</v>
+        <v>35</v>
       </c>
       <c r="H233" s="17" t="s">
         <v>37</v>
@@ -9405,7 +9405,7 @@
         <v>36</v>
       </c>
       <c r="G234" s="19">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="H234" s="17" t="s">
         <v>37</v>
@@ -9431,7 +9431,7 @@
         <v>36</v>
       </c>
       <c r="G235" s="19">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="H235" s="17" t="s">
         <v>37</v>
@@ -9457,7 +9457,7 @@
         <v>36</v>
       </c>
       <c r="G236" s="19">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="H236" s="17" t="s">
         <v>37</v>
@@ -9483,7 +9483,7 @@
         <v>36</v>
       </c>
       <c r="G237" s="19">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H237" s="17" t="s">
         <v>37</v>
@@ -9509,7 +9509,7 @@
         <v>36</v>
       </c>
       <c r="G238" s="19">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="H238" s="17" t="s">
         <v>37</v>
@@ -9535,7 +9535,7 @@
         <v>36</v>
       </c>
       <c r="G239" s="19">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="H239" s="17" t="s">
         <v>37</v>
@@ -9561,7 +9561,7 @@
         <v>36</v>
       </c>
       <c r="G240" s="19">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="H240" s="17" t="s">
         <v>37</v>
@@ -9587,7 +9587,7 @@
         <v>36</v>
       </c>
       <c r="G241" s="19">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="H241" s="17" t="s">
         <v>37</v>
@@ -9613,7 +9613,7 @@
         <v>36</v>
       </c>
       <c r="G242" s="19">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="H242" s="17" t="s">
         <v>37</v>
@@ -9639,7 +9639,7 @@
         <v>36</v>
       </c>
       <c r="G243" s="19">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="H243" s="17" t="s">
         <v>37</v>
@@ -9665,7 +9665,7 @@
         <v>36</v>
       </c>
       <c r="G244" s="19">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="H244" s="17" t="s">
         <v>37</v>
@@ -9691,7 +9691,7 @@
         <v>36</v>
       </c>
       <c r="G245" s="19">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="H245" s="17" t="s">
         <v>37</v>
@@ -9717,7 +9717,7 @@
         <v>36</v>
       </c>
       <c r="G246" s="19">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="H246" s="17" t="s">
         <v>37</v>
@@ -9743,7 +9743,7 @@
         <v>36</v>
       </c>
       <c r="G247" s="19">
-        <v>20</v>
+        <v>3</v>
       </c>
       <c r="H247" s="17" t="s">
         <v>37</v>
@@ -9769,7 +9769,7 @@
         <v>36</v>
       </c>
       <c r="G248" s="19">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="H248" s="17" t="s">
         <v>37</v>
@@ -9795,7 +9795,7 @@
         <v>36</v>
       </c>
       <c r="G249" s="19">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="H249" s="17" t="s">
         <v>37</v>
@@ -9821,7 +9821,7 @@
         <v>36</v>
       </c>
       <c r="G250" s="19">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H250" s="17" t="s">
         <v>37</v>
@@ -9847,7 +9847,7 @@
         <v>36</v>
       </c>
       <c r="G251" s="19">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H251" s="17" t="s">
         <v>37</v>
@@ -9873,7 +9873,7 @@
         <v>36</v>
       </c>
       <c r="G252" s="19">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="H252" s="17" t="s">
         <v>37</v>
@@ -9899,7 +9899,7 @@
         <v>36</v>
       </c>
       <c r="G253" s="19">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H253" s="17" t="s">
         <v>37</v>
@@ -9925,7 +9925,7 @@
         <v>36</v>
       </c>
       <c r="G254" s="19">
-        <v>12</v>
+        <v>34</v>
       </c>
       <c r="H254" s="17" t="s">
         <v>37</v>
@@ -9951,7 +9951,7 @@
         <v>36</v>
       </c>
       <c r="G255" s="19">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="H255" s="17" t="s">
         <v>37</v>
@@ -9977,7 +9977,7 @@
         <v>36</v>
       </c>
       <c r="G256" s="19">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="H256" s="17" t="s">
         <v>37</v>
@@ -10003,7 +10003,7 @@
         <v>36</v>
       </c>
       <c r="G257" s="19">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H257" s="17" t="s">
         <v>37</v>
@@ -10029,7 +10029,7 @@
         <v>36</v>
       </c>
       <c r="G258" s="19">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="H258" s="17" t="s">
         <v>37</v>
@@ -10055,7 +10055,7 @@
         <v>36</v>
       </c>
       <c r="G259" s="19">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="H259" s="17" t="s">
         <v>37</v>
@@ -10081,7 +10081,7 @@
         <v>36</v>
       </c>
       <c r="G260" s="19">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H260" s="17" t="s">
         <v>37</v>
@@ -10107,7 +10107,7 @@
         <v>36</v>
       </c>
       <c r="G261" s="19">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="H261" s="17" t="s">
         <v>37</v>
@@ -10133,7 +10133,7 @@
         <v>36</v>
       </c>
       <c r="G262" s="19">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H262" s="17" t="s">
         <v>37</v>
@@ -10159,7 +10159,7 @@
         <v>36</v>
       </c>
       <c r="G263" s="19">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="H263" s="17" t="s">
         <v>37</v>
@@ -10185,7 +10185,7 @@
         <v>36</v>
       </c>
       <c r="G264" s="19">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="H264" s="17" t="s">
         <v>37</v>
@@ -10211,7 +10211,7 @@
         <v>36</v>
       </c>
       <c r="G265" s="19">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="H265" s="17" t="s">
         <v>37</v>
@@ -10237,7 +10237,7 @@
         <v>36</v>
       </c>
       <c r="G266" s="19">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="H266" s="17" t="s">
         <v>37</v>
@@ -10263,7 +10263,7 @@
         <v>36</v>
       </c>
       <c r="G267" s="19">
-        <v>7</v>
+        <v>34</v>
       </c>
       <c r="H267" s="17" t="s">
         <v>37</v>
@@ -10289,7 +10289,7 @@
         <v>36</v>
       </c>
       <c r="G268" s="19">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="H268" s="17" t="s">
         <v>37</v>
@@ -10315,7 +10315,7 @@
         <v>36</v>
       </c>
       <c r="G269" s="19">
-        <v>31</v>
+        <v>3</v>
       </c>
       <c r="H269" s="17" t="s">
         <v>37</v>
@@ -10341,7 +10341,7 @@
         <v>36</v>
       </c>
       <c r="G270" s="19">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="H270" s="17" t="s">
         <v>37</v>
@@ -10367,7 +10367,7 @@
         <v>36</v>
       </c>
       <c r="G271" s="19">
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="H271" s="17" t="s">
         <v>37</v>
@@ -10393,7 +10393,7 @@
         <v>36</v>
       </c>
       <c r="G272" s="19">
-        <v>8</v>
+        <v>27</v>
       </c>
       <c r="H272" s="17" t="s">
         <v>37</v>
@@ -10419,7 +10419,7 @@
         <v>36</v>
       </c>
       <c r="G273" s="19">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H273" s="17" t="s">
         <v>37</v>
@@ -10445,7 +10445,7 @@
         <v>36</v>
       </c>
       <c r="G274" s="19">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H274" s="17" t="s">
         <v>37</v>
@@ -10471,7 +10471,7 @@
         <v>36</v>
       </c>
       <c r="G275" s="19">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="H275" s="17" t="s">
         <v>37</v>
@@ -10497,7 +10497,7 @@
         <v>36</v>
       </c>
       <c r="G276" s="19">
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H276" s="17" t="s">
         <v>37</v>
@@ -10523,7 +10523,7 @@
         <v>36</v>
       </c>
       <c r="G277" s="19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H277" s="17" t="s">
         <v>37</v>
@@ -10549,7 +10549,7 @@
         <v>36</v>
       </c>
       <c r="G278" s="19">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H278" s="17" t="s">
         <v>37</v>
@@ -10575,7 +10575,7 @@
         <v>36</v>
       </c>
       <c r="G279" s="19">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="H279" s="17" t="s">
         <v>37</v>
@@ -10627,7 +10627,7 @@
         <v>36</v>
       </c>
       <c r="G281" s="19">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="H281" s="17" t="s">
         <v>37</v>
@@ -10653,7 +10653,7 @@
         <v>36</v>
       </c>
       <c r="G282" s="19">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="H282" s="17" t="s">
         <v>37</v>
@@ -10705,7 +10705,7 @@
         <v>36</v>
       </c>
       <c r="G284" s="19">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H284" s="17" t="s">
         <v>37</v>
@@ -10731,7 +10731,7 @@
         <v>36</v>
       </c>
       <c r="G285" s="19">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="H285" s="17" t="s">
         <v>37</v>
@@ -10757,7 +10757,7 @@
         <v>36</v>
       </c>
       <c r="G286" s="19">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="H286" s="17" t="s">
         <v>37</v>
@@ -10783,7 +10783,7 @@
         <v>36</v>
       </c>
       <c r="G287" s="19">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="H287" s="17" t="s">
         <v>37</v>
@@ -10809,7 +10809,7 @@
         <v>36</v>
       </c>
       <c r="G288" s="19">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="H288" s="17" t="s">
         <v>37</v>
@@ -10835,7 +10835,7 @@
         <v>36</v>
       </c>
       <c r="G289" s="19">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="H289" s="17" t="s">
         <v>37</v>
@@ -10861,7 +10861,7 @@
         <v>36</v>
       </c>
       <c r="G290" s="19">
-        <v>22</v>
+        <v>37</v>
       </c>
       <c r="H290" s="17" t="s">
         <v>37</v>
@@ -10887,7 +10887,7 @@
         <v>36</v>
       </c>
       <c r="G291" s="19">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="H291" s="17" t="s">
         <v>37</v>
@@ -10913,7 +10913,7 @@
         <v>36</v>
       </c>
       <c r="G292" s="19">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="H292" s="17" t="s">
         <v>37</v>
@@ -10939,7 +10939,7 @@
         <v>36</v>
       </c>
       <c r="G293" s="19">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H293" s="17" t="s">
         <v>37</v>
@@ -10965,7 +10965,7 @@
         <v>36</v>
       </c>
       <c r="G294" s="19">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="H294" s="17" t="s">
         <v>37</v>
@@ -10991,7 +10991,7 @@
         <v>36</v>
       </c>
       <c r="G295" s="19">
-        <v>2</v>
+        <v>37</v>
       </c>
       <c r="H295" s="17" t="s">
         <v>37</v>
@@ -11017,7 +11017,7 @@
         <v>36</v>
       </c>
       <c r="G296" s="19">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="H296" s="17" t="s">
         <v>37</v>
@@ -11043,7 +11043,7 @@
         <v>36</v>
       </c>
       <c r="G297" s="19">
-        <v>3</v>
+        <v>25</v>
       </c>
       <c r="H297" s="17" t="s">
         <v>37</v>
@@ -11069,7 +11069,7 @@
         <v>36</v>
       </c>
       <c r="G298" s="19">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H298" s="17" t="s">
         <v>37</v>
@@ -11095,7 +11095,7 @@
         <v>36</v>
       </c>
       <c r="G299" s="19">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H299" s="17" t="s">
         <v>37</v>
@@ -11121,7 +11121,7 @@
         <v>36</v>
       </c>
       <c r="G300" s="19">
-        <v>18</v>
+        <v>39</v>
       </c>
       <c r="H300" s="17" t="s">
         <v>37</v>
@@ -11147,7 +11147,7 @@
         <v>36</v>
       </c>
       <c r="G301" s="19">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="H301" s="17" t="s">
         <v>37</v>
@@ -11173,7 +11173,7 @@
         <v>36</v>
       </c>
       <c r="G302" s="19">
-        <v>9</v>
+        <v>38</v>
       </c>
       <c r="H302" s="17" t="s">
         <v>37</v>
@@ -11199,7 +11199,7 @@
         <v>36</v>
       </c>
       <c r="G303" s="19">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="H303" s="17" t="s">
         <v>37</v>
@@ -11225,7 +11225,7 @@
         <v>36</v>
       </c>
       <c r="G304" s="19">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="H304" s="17" t="s">
         <v>37</v>
@@ -11251,7 +11251,7 @@
         <v>36</v>
       </c>
       <c r="G305" s="19">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H305" s="17" t="s">
         <v>37</v>
@@ -11277,7 +11277,7 @@
         <v>36</v>
       </c>
       <c r="G306" s="19">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="H306" s="17" t="s">
         <v>37</v>
@@ -11303,7 +11303,7 @@
         <v>36</v>
       </c>
       <c r="G307" s="19">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H307" s="17" t="s">
         <v>37</v>
@@ -11329,7 +11329,7 @@
         <v>36</v>
       </c>
       <c r="G308" s="19">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H308" s="17" t="s">
         <v>37</v>
@@ -11355,7 +11355,7 @@
         <v>36</v>
       </c>
       <c r="G309" s="19">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H309" s="17" t="s">
         <v>37</v>
@@ -11381,7 +11381,7 @@
         <v>36</v>
       </c>
       <c r="G310" s="19">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="H310" s="17" t="s">
         <v>37</v>
@@ -11407,7 +11407,7 @@
         <v>36</v>
       </c>
       <c r="G311" s="19">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="H311" s="17" t="s">
         <v>37</v>
@@ -11433,7 +11433,7 @@
         <v>36</v>
       </c>
       <c r="G312" s="19">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="H312" s="17" t="s">
         <v>37</v>
@@ -11459,7 +11459,7 @@
         <v>36</v>
       </c>
       <c r="G313" s="19">
-        <v>25</v>
+        <v>11</v>
       </c>
       <c r="H313" s="17" t="s">
         <v>37</v>
@@ -11485,7 +11485,7 @@
         <v>36</v>
       </c>
       <c r="G314" s="19">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="H314" s="17" t="s">
         <v>37</v>
@@ -11511,7 +11511,7 @@
         <v>36</v>
       </c>
       <c r="G315" s="19">
-        <v>3</v>
+        <v>34</v>
       </c>
       <c r="H315" s="17" t="s">
         <v>37</v>
@@ -11537,7 +11537,7 @@
         <v>36</v>
       </c>
       <c r="G316" s="19">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H316" s="17" t="s">
         <v>37</v>
@@ -11563,7 +11563,7 @@
         <v>36</v>
       </c>
       <c r="G317" s="19">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="H317" s="17" t="s">
         <v>37</v>
@@ -11589,7 +11589,7 @@
         <v>36</v>
       </c>
       <c r="G318" s="19">
-        <v>39</v>
+        <v>9</v>
       </c>
       <c r="H318" s="17" t="s">
         <v>37</v>
@@ -11615,7 +11615,7 @@
         <v>36</v>
       </c>
       <c r="G319" s="19">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="H319" s="17" t="s">
         <v>37</v>
@@ -11641,7 +11641,7 @@
         <v>36</v>
       </c>
       <c r="G320" s="19">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H320" s="17" t="s">
         <v>37</v>
@@ -11667,7 +11667,7 @@
         <v>36</v>
       </c>
       <c r="G321" s="19">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="H321" s="17" t="s">
         <v>37</v>
@@ -11693,7 +11693,7 @@
         <v>36</v>
       </c>
       <c r="G322" s="19">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="H322" s="17" t="s">
         <v>37</v>
@@ -11719,7 +11719,7 @@
         <v>36</v>
       </c>
       <c r="G323" s="19">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H323" s="17" t="s">
         <v>37</v>
@@ -11745,7 +11745,7 @@
         <v>36</v>
       </c>
       <c r="G324" s="19">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="H324" s="17" t="s">
         <v>37</v>
@@ -11771,7 +11771,7 @@
         <v>36</v>
       </c>
       <c r="G325" s="19">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="H325" s="17" t="s">
         <v>37</v>
@@ -11797,7 +11797,7 @@
         <v>36</v>
       </c>
       <c r="G326" s="19">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="H326" s="17" t="s">
         <v>37</v>
@@ -11823,7 +11823,7 @@
         <v>36</v>
       </c>
       <c r="G327" s="19">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="H327" s="17" t="s">
         <v>37</v>
@@ -11849,7 +11849,7 @@
         <v>36</v>
       </c>
       <c r="G328" s="19">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H328" s="17" t="s">
         <v>37</v>
@@ -11875,7 +11875,7 @@
         <v>36</v>
       </c>
       <c r="G329" s="19">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="H329" s="17" t="s">
         <v>37</v>
@@ -11901,7 +11901,7 @@
         <v>36</v>
       </c>
       <c r="G330" s="19">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H330" s="17" t="s">
         <v>37</v>
@@ -11927,7 +11927,7 @@
         <v>36</v>
       </c>
       <c r="G331" s="19">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="H331" s="17" t="s">
         <v>37</v>
@@ -11953,7 +11953,7 @@
         <v>36</v>
       </c>
       <c r="G332" s="19">
-        <v>30</v>
+        <v>3</v>
       </c>
       <c r="H332" s="17" t="s">
         <v>37</v>
@@ -11979,7 +11979,7 @@
         <v>36</v>
       </c>
       <c r="G333" s="19">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="H333" s="17" t="s">
         <v>37</v>
@@ -12005,7 +12005,7 @@
         <v>36</v>
       </c>
       <c r="G334" s="19">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H334" s="17" t="s">
         <v>37</v>
@@ -12031,7 +12031,7 @@
         <v>36</v>
       </c>
       <c r="G335" s="19">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="H335" s="17" t="s">
         <v>37</v>
@@ -12057,7 +12057,7 @@
         <v>36</v>
       </c>
       <c r="G336" s="19">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="H336" s="17" t="s">
         <v>37</v>
@@ -12083,7 +12083,7 @@
         <v>36</v>
       </c>
       <c r="G337" s="19">
-        <v>37</v>
+        <v>0</v>
       </c>
       <c r="H337" s="17" t="s">
         <v>37</v>
@@ -12109,7 +12109,7 @@
         <v>36</v>
       </c>
       <c r="G338" s="19">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="H338" s="17" t="s">
         <v>37</v>
@@ -12135,7 +12135,7 @@
         <v>36</v>
       </c>
       <c r="G339" s="19">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="H339" s="17" t="s">
         <v>37</v>
@@ -12187,7 +12187,7 @@
         <v>36</v>
       </c>
       <c r="G341" s="19">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="H341" s="17" t="s">
         <v>37</v>
@@ -12213,7 +12213,7 @@
         <v>36</v>
       </c>
       <c r="G342" s="19">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H342" s="17" t="s">
         <v>37</v>
@@ -12239,7 +12239,7 @@
         <v>36</v>
       </c>
       <c r="G343" s="19">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="H343" s="17" t="s">
         <v>37</v>
@@ -12265,7 +12265,7 @@
         <v>36</v>
       </c>
       <c r="G344" s="19">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="H344" s="17" t="s">
         <v>37</v>
@@ -12291,7 +12291,7 @@
         <v>36</v>
       </c>
       <c r="G345" s="19">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="H345" s="17" t="s">
         <v>37</v>
@@ -12317,7 +12317,7 @@
         <v>36</v>
       </c>
       <c r="G346" s="19">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="H346" s="17" t="s">
         <v>37</v>
@@ -12343,7 +12343,7 @@
         <v>36</v>
       </c>
       <c r="G347" s="19">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H347" s="17" t="s">
         <v>37</v>
@@ -12369,7 +12369,7 @@
         <v>36</v>
       </c>
       <c r="G348" s="19">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H348" s="17" t="s">
         <v>37</v>
@@ -12395,7 +12395,7 @@
         <v>36</v>
       </c>
       <c r="G349" s="19">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H349" s="17" t="s">
         <v>37</v>
@@ -12421,7 +12421,7 @@
         <v>36</v>
       </c>
       <c r="G350" s="19">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="H350" s="17" t="s">
         <v>37</v>
@@ -12447,7 +12447,7 @@
         <v>36</v>
       </c>
       <c r="G351" s="19">
-        <v>6</v>
+        <v>34</v>
       </c>
       <c r="H351" s="17" t="s">
         <v>37</v>
@@ -12473,7 +12473,7 @@
         <v>36</v>
       </c>
       <c r="G352" s="19">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="H352" s="17" t="s">
         <v>37</v>
@@ -12499,7 +12499,7 @@
         <v>36</v>
       </c>
       <c r="G353" s="19">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H353" s="17" t="s">
         <v>37</v>
@@ -12525,7 +12525,7 @@
         <v>36</v>
       </c>
       <c r="G354" s="19">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="H354" s="17" t="s">
         <v>37</v>
@@ -12551,7 +12551,7 @@
         <v>36</v>
       </c>
       <c r="G355" s="19">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="H355" s="17" t="s">
         <v>37</v>
@@ -12577,7 +12577,7 @@
         <v>36</v>
       </c>
       <c r="G356" s="19">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="H356" s="17" t="s">
         <v>37</v>
@@ -12603,7 +12603,7 @@
         <v>36</v>
       </c>
       <c r="G357" s="19">
-        <v>37</v>
+        <v>13</v>
       </c>
       <c r="H357" s="17" t="s">
         <v>37</v>
@@ -12629,7 +12629,7 @@
         <v>36</v>
       </c>
       <c r="G358" s="19">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="H358" s="17" t="s">
         <v>37</v>
@@ -12655,7 +12655,7 @@
         <v>36</v>
       </c>
       <c r="G359" s="19">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="H359" s="17" t="s">
         <v>37</v>
@@ -12681,7 +12681,7 @@
         <v>36</v>
       </c>
       <c r="G360" s="19">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="H360" s="17" t="s">
         <v>37</v>
@@ -12707,7 +12707,7 @@
         <v>36</v>
       </c>
       <c r="G361" s="19">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H361" s="17" t="s">
         <v>37</v>
@@ -12733,7 +12733,7 @@
         <v>36</v>
       </c>
       <c r="G362" s="19">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="H362" s="17" t="s">
         <v>37</v>
@@ -12759,7 +12759,7 @@
         <v>36</v>
       </c>
       <c r="G363" s="19">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="H363" s="17" t="s">
         <v>37</v>
@@ -12785,7 +12785,7 @@
         <v>36</v>
       </c>
       <c r="G364" s="19">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="H364" s="17" t="s">
         <v>37</v>
@@ -12811,7 +12811,7 @@
         <v>36</v>
       </c>
       <c r="G365" s="19">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="H365" s="17" t="s">
         <v>37</v>
@@ -12837,7 +12837,7 @@
         <v>36</v>
       </c>
       <c r="G366" s="19">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="H366" s="17" t="s">
         <v>37</v>
@@ -12863,7 +12863,7 @@
         <v>36</v>
       </c>
       <c r="G367" s="19">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H367" s="17" t="s">
         <v>37</v>
@@ -12889,7 +12889,7 @@
         <v>36</v>
       </c>
       <c r="G368" s="19">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H368" s="17" t="s">
         <v>37</v>
@@ -12915,7 +12915,7 @@
         <v>36</v>
       </c>
       <c r="G369" s="19">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="H369" s="17" t="s">
         <v>37</v>
@@ -12941,7 +12941,7 @@
         <v>36</v>
       </c>
       <c r="G370" s="19">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H370" s="17" t="s">
         <v>37</v>
@@ -12967,7 +12967,7 @@
         <v>36</v>
       </c>
       <c r="G371" s="19">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="H371" s="17" t="s">
         <v>37</v>
@@ -12993,7 +12993,7 @@
         <v>36</v>
       </c>
       <c r="G372" s="19">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="H372" s="17" t="s">
         <v>37</v>
@@ -13019,7 +13019,7 @@
         <v>36</v>
       </c>
       <c r="G373" s="19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H373" s="17" t="s">
         <v>37</v>
@@ -13045,7 +13045,7 @@
         <v>36</v>
       </c>
       <c r="G374" s="19">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="H374" s="17" t="s">
         <v>37</v>
@@ -13097,7 +13097,7 @@
         <v>36</v>
       </c>
       <c r="G376" s="19">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H376" s="17" t="s">
         <v>37</v>
@@ -13123,7 +13123,7 @@
         <v>36</v>
       </c>
       <c r="G377" s="19">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="H377" s="17" t="s">
         <v>37</v>
@@ -13149,7 +13149,7 @@
         <v>36</v>
       </c>
       <c r="G378" s="19">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="H378" s="17" t="s">
         <v>37</v>
@@ -13175,7 +13175,7 @@
         <v>36</v>
       </c>
       <c r="G379" s="19">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H379" s="17" t="s">
         <v>37</v>
@@ -13201,7 +13201,7 @@
         <v>36</v>
       </c>
       <c r="G380" s="19">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H380" s="17" t="s">
         <v>37</v>
@@ -13227,7 +13227,7 @@
         <v>36</v>
       </c>
       <c r="G381" s="19">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="H381" s="17" t="s">
         <v>37</v>
@@ -13253,7 +13253,7 @@
         <v>36</v>
       </c>
       <c r="G382" s="19">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="H382" s="17" t="s">
         <v>37</v>
@@ -13279,7 +13279,7 @@
         <v>36</v>
       </c>
       <c r="G383" s="19">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="H383" s="17" t="s">
         <v>37</v>
@@ -13305,7 +13305,7 @@
         <v>36</v>
       </c>
       <c r="G384" s="19">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H384" s="17" t="s">
         <v>37</v>
@@ -13331,7 +13331,7 @@
         <v>36</v>
       </c>
       <c r="G385" s="19">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H385" s="17" t="s">
         <v>37</v>
@@ -13357,7 +13357,7 @@
         <v>36</v>
       </c>
       <c r="G386" s="19">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="H386" s="17" t="s">
         <v>37</v>
@@ -13383,7 +13383,7 @@
         <v>36</v>
       </c>
       <c r="G387" s="19">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="H387" s="17" t="s">
         <v>37</v>
@@ -13409,7 +13409,7 @@
         <v>36</v>
       </c>
       <c r="G388" s="19">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="H388" s="17" t="s">
         <v>37</v>
@@ -13435,7 +13435,7 @@
         <v>36</v>
       </c>
       <c r="G389" s="19">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="H389" s="17" t="s">
         <v>37</v>
@@ -13461,7 +13461,7 @@
         <v>36</v>
       </c>
       <c r="G390" s="19">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H390" s="17" t="s">
         <v>37</v>
@@ -13487,7 +13487,7 @@
         <v>36</v>
       </c>
       <c r="G391" s="19">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="H391" s="17" t="s">
         <v>37</v>
@@ -13539,7 +13539,7 @@
         <v>36</v>
       </c>
       <c r="G393" s="19">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="H393" s="17" t="s">
         <v>37</v>
@@ -13565,7 +13565,7 @@
         <v>36</v>
       </c>
       <c r="G394" s="19">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="H394" s="17" t="s">
         <v>37</v>
@@ -13591,7 +13591,7 @@
         <v>36</v>
       </c>
       <c r="G395" s="19">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="H395" s="17" t="s">
         <v>37</v>
@@ -13617,7 +13617,7 @@
         <v>36</v>
       </c>
       <c r="G396" s="19">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H396" s="17" t="s">
         <v>37</v>
@@ -13643,7 +13643,7 @@
         <v>36</v>
       </c>
       <c r="G397" s="19">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="H397" s="17" t="s">
         <v>37</v>
@@ -13669,7 +13669,7 @@
         <v>36</v>
       </c>
       <c r="G398" s="19">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="H398" s="17" t="s">
         <v>37</v>
@@ -13695,7 +13695,7 @@
         <v>36</v>
       </c>
       <c r="G399" s="19">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="H399" s="17" t="s">
         <v>37</v>
@@ -13721,7 +13721,7 @@
         <v>36</v>
       </c>
       <c r="G400" s="19">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="H400" s="17" t="s">
         <v>37</v>
@@ -13747,7 +13747,7 @@
         <v>36</v>
       </c>
       <c r="G401" s="19">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H401" s="17" t="s">
         <v>37</v>

</xml_diff>